<commit_message>
Armand (Pfarre Koppl): 200 kg Birnen + 150 kg Zwetschken za 1,25
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBB3165-CBC1-432F-81A6-81D169BC028D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B3816D-D299-4E44-AA1E-B9C9D0520F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1610,14 +1610,14 @@
         <v>77</v>
       </c>
       <c r="C35" s="9">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="D35" s="9">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="E35" s="9">
         <f t="shared" si="1"/>
-        <v>130</v>
+        <v>187.5</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>78</v>
@@ -1947,14 +1947,14 @@
         <v>77</v>
       </c>
       <c r="C49" s="9">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D49" s="9">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="E49" s="9">
         <f t="shared" si="2"/>
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>78</v>
@@ -2053,12 +2053,12 @@
       </c>
       <c r="C54" s="3">
         <f>SUM(C2:C53)</f>
-        <v>25000</v>
+        <v>25150</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" s="8">
         <f>SUM(E2:E53)</f>
-        <v>32160</v>
+        <v>32347.5</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova objednavka: Burgstaller 1000 kg Birnen Packham za 1,10 (novy blok)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B3816D-D299-4E44-AA1E-B9C9D0520F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="105">
   <si>
     <t>Geliefert</t>
   </si>
@@ -324,6 +324,9 @@
   </si>
   <si>
     <t>(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
+  </si>
+  <si>
+    <t>Birnen Packham</t>
   </si>
   <si>
     <t>Äpfel</t>
@@ -784,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1998,78 +2001,103 @@
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="C52" s="9">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="D52" s="9">
-        <v>0.7</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E52" s="9">
         <f>C52*D52</f>
+        <v>1100</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A53" s="9"/>
+      <c r="B53" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A54" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C54" s="9">
+        <v>400</v>
+      </c>
+      <c r="D54" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="E54" s="9">
+        <f>C54*D54</f>
         <v>280</v>
       </c>
-      <c r="F52" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="G52" s="9" t="s">
+      <c r="F54" s="9" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="B53" s="9" t="s">
+      <c r="G54" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="C53" s="9">
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A55" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C55" s="9">
         <v>300</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D55" s="9">
         <v>0.75</v>
       </c>
-      <c r="E53" s="9">
-        <f>C53*D53</f>
+      <c r="E55" s="9">
+        <f>C55*D55</f>
         <v>225</v>
       </c>
-      <c r="F53" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="G53" s="9" t="s">
+      <c r="F55" s="9" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" t="b">
-        <v>0</v>
-      </c>
-      <c r="C54" s="3">
-        <f>SUM(C2:C53)</f>
-        <v>25150</v>
-      </c>
-      <c r="D54" s="3"/>
-      <c r="E54" s="8">
-        <f>SUM(E2:E53)</f>
-        <v>32347.5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A55" t="b">
-        <v>0</v>
+      <c r="G55" s="9" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="b">
         <v>0</v>
       </c>
+      <c r="C56" s="3">
+        <f>SUM(C2:C55)</f>
+        <v>26150</v>
+      </c>
+      <c r="D56" s="3"/>
+      <c r="E56" s="8">
+        <f>SUM(E2:E55)</f>
+        <v>33447.5</v>
+      </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="b">
@@ -2148,6 +2176,16 @@
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fuchs Freund (Pfarrer): adresa Pfarramt Thalgau, Pfarrhofallee 7
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03FB7357-EBF3-46A5-8D81-9BF4672ECFE5}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="106">
   <si>
     <t>Geliefert</t>
   </si>
@@ -194,9 +194,6 @@
     <t>Fuchs Freund</t>
   </si>
   <si>
-    <t>Lämmererweg 2 5321 Koppl</t>
-  </si>
-  <si>
     <t>Herz Jesu</t>
   </si>
   <si>
@@ -348,6 +345,12 @@
   </si>
   <si>
     <t>(47.2765915, 13.3198029)</t>
+  </si>
+  <si>
+    <t>Pfarramt Thalgau, Pfarrhofallee 7, 5303 Thalgau</t>
+  </si>
+  <si>
+    <t>Pfarrer, Freund von Peter Fuchs – Übergabe in Koppl</t>
   </si>
 </sst>
 </file>
@@ -355,9 +358,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
-    <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -425,21 +428,21 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -1352,7 +1355,10 @@
         <v>150</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>53</v>
+        <v>104</v>
+      </c>
+      <c r="G23" t="s">
+        <v>105</v>
       </c>
       <c r="H23" s="10">
         <v>46222</v>
@@ -1363,7 +1369,7 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C24" s="3">
         <v>360</v>
@@ -1377,10 +1383,10 @@
         <v>400</v>
       </c>
       <c r="F24" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" t="s">
         <v>55</v>
-      </c>
-      <c r="G24" t="s">
-        <v>56</v>
       </c>
       <c r="H24" s="10">
         <v>46222</v>
@@ -1391,7 +1397,7 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C25">
         <v>950</v>
@@ -1404,10 +1410,10 @@
         <v>1425</v>
       </c>
       <c r="F25" t="s">
+        <v>57</v>
+      </c>
+      <c r="G25" t="s">
         <v>58</v>
-      </c>
-      <c r="G25" t="s">
-        <v>59</v>
       </c>
       <c r="H25" s="10">
         <v>46233</v>
@@ -1418,7 +1424,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="9">
         <v>300</v>
@@ -1431,7 +1437,7 @@
         <v>450</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G26" s="9"/>
       <c r="H26" s="10">
@@ -1443,7 +1449,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C27" s="9">
         <v>1000</v>
@@ -1456,7 +1462,7 @@
         <v>1500</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G27" s="9"/>
       <c r="H27" s="10">
@@ -1468,7 +1474,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C28" s="9">
         <v>300</v>
@@ -1481,7 +1487,7 @@
         <v>450</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G28" s="9"/>
       <c r="H28" s="10">
@@ -1498,7 +1504,7 @@
         <v>0</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -1511,7 +1517,7 @@
         <v>0</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C31" s="9">
         <v>0</v>
@@ -1519,10 +1525,10 @@
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G31" s="9" t="s">
         <v>68</v>
-      </c>
-      <c r="G31" s="9" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -1530,7 +1536,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C32" s="9">
         <v>380</v>
@@ -1544,10 +1550,10 @@
         <v>350</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H32" s="10">
         <v>46271</v>
@@ -1558,7 +1564,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C33" s="9">
         <v>260</v>
@@ -1572,10 +1578,10 @@
         <v>290</v>
       </c>
       <c r="F33" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>73</v>
       </c>
       <c r="H33" s="10">
         <v>46271</v>
@@ -1586,7 +1592,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C34" s="9">
         <v>300</v>
@@ -1599,10 +1605,10 @@
         <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G34" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -1610,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C35" s="9">
         <v>150</v>
@@ -1623,10 +1629,10 @@
         <v>187.5</v>
       </c>
       <c r="F35" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="G35" s="9" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
@@ -1709,7 +1715,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C39" s="9">
         <v>300</v>
@@ -1722,7 +1728,7 @@
         <v>330</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="10">
@@ -1750,7 +1756,7 @@
         <v>31</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
@@ -1758,7 +1764,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C41" s="9">
         <v>400</v>
@@ -1771,10 +1777,10 @@
         <v>520</v>
       </c>
       <c r="F41" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G41" s="9" t="s">
         <v>84</v>
-      </c>
-      <c r="G41" s="9" t="s">
-        <v>85</v>
       </c>
       <c r="H41" s="10">
         <v>46271</v>
@@ -1801,7 +1807,7 @@
         <v>23</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H42" s="10">
         <v>46273</v>
@@ -1812,7 +1818,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C43" s="9">
         <v>500</v>
@@ -1825,7 +1831,7 @@
         <v>475</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G43" s="9"/>
       <c r="H43" s="10">
@@ -1837,7 +1843,7 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -1863,7 +1869,7 @@
         <v>1200</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G45" s="9"/>
     </row>
@@ -1888,7 +1894,7 @@
         <v>44</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H46" s="10">
         <v>46273</v>
@@ -1899,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C47" s="9">
         <v>600</v>
@@ -1912,10 +1918,10 @@
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G47" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -1923,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C48" s="9">
         <v>300</v>
@@ -1936,10 +1942,10 @@
         <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
@@ -1947,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C49" s="9">
         <v>200</v>
@@ -1960,10 +1966,10 @@
         <v>250</v>
       </c>
       <c r="F49" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G49" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
@@ -1987,14 +1993,14 @@
         <v>23</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="9"/>
       <c r="B51" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
@@ -2029,7 +2035,7 @@
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="9"/>
       <c r="B53" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
@@ -2042,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C54" s="9">
         <v>400</v>
@@ -2055,10 +2061,10 @@
         <v>280</v>
       </c>
       <c r="F54" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G54" s="9" t="s">
         <v>100</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
@@ -2066,7 +2072,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C55" s="9">
         <v>300</v>
@@ -2079,10 +2085,10 @@
         <v>225</v>
       </c>
       <c r="F55" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G55" s="9" t="s">
         <v>103</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Fuchs Freund (Pfarrer): adresa jen Pfarramt Thalgau + GPS
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03FB7357-EBF3-46A5-8D81-9BF4672ECFE5}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16EB54B7-D83D-47EB-86C1-901A8BB1E551}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -347,10 +347,10 @@
     <t>(47.2765915, 13.3198029)</t>
   </si>
   <si>
-    <t>Pfarramt Thalgau, Pfarrhofallee 7, 5303 Thalgau</t>
-  </si>
-  <si>
-    <t>Pfarrer, Freund von Peter Fuchs – Übergabe in Koppl</t>
+    <t>Pfarramt Thalgau</t>
+  </si>
+  <si>
+    <t>(47.8450105, 13.2584452) Pfarrer, Freund von Peter Fuchs – Übergabe in Koppl</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Armand (farar): vsechny radky Pfarramt Thalgau + GPS, Fuchs Freund prejmenovan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16EB54B7-D83D-47EB-86C1-901A8BB1E551}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C47A436-D14B-4234-825F-F5BA19FA1475}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="104">
   <si>
     <t>Geliefert</t>
   </si>
@@ -191,9 +191,6 @@
     <t>Lämmererweg 2 5321 Koppl </t>
   </si>
   <si>
-    <t>Fuchs Freund</t>
-  </si>
-  <si>
     <t>Herz Jesu</t>
   </si>
   <si>
@@ -266,12 +263,6 @@
     <t>Armand, Pfarre Koppl</t>
   </si>
   <si>
-    <t>5321 Koppl</t>
-  </si>
-  <si>
-    <t>(47.8081289, 13.1570363) Pfarre (bei der Pfarrkirche, Dorfstraße)</t>
-  </si>
-  <si>
     <t>Rainer</t>
   </si>
   <si>
@@ -350,7 +341,10 @@
     <t>Pfarramt Thalgau</t>
   </si>
   <si>
-    <t>(47.8450105, 13.2584452) Pfarrer, Freund von Peter Fuchs – Übergabe in Koppl</t>
+    <t>(47.8450105, 13.2584452) Übergabe in Koppl bei Peter Fuchs</t>
+  </si>
+  <si>
+    <t>(47.8450105, 13.2584452)</t>
   </si>
 </sst>
 </file>
@@ -1342,7 +1336,7 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C23" s="3">
         <v>100</v>
@@ -1355,10 +1349,10 @@
         <v>150</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G23" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H23" s="10">
         <v>46222</v>
@@ -1369,7 +1363,7 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C24" s="3">
         <v>360</v>
@@ -1383,10 +1377,10 @@
         <v>400</v>
       </c>
       <c r="F24" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G24" t="s">
         <v>54</v>
-      </c>
-      <c r="G24" t="s">
-        <v>55</v>
       </c>
       <c r="H24" s="10">
         <v>46222</v>
@@ -1397,7 +1391,7 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
         <v>950</v>
@@ -1410,10 +1404,10 @@
         <v>1425</v>
       </c>
       <c r="F25" t="s">
+        <v>56</v>
+      </c>
+      <c r="G25" t="s">
         <v>57</v>
-      </c>
-      <c r="G25" t="s">
-        <v>58</v>
       </c>
       <c r="H25" s="10">
         <v>46233</v>
@@ -1424,7 +1418,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26" s="9">
         <v>300</v>
@@ -1437,7 +1431,7 @@
         <v>450</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G26" s="9"/>
       <c r="H26" s="10">
@@ -1449,7 +1443,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C27" s="9">
         <v>1000</v>
@@ -1462,7 +1456,7 @@
         <v>1500</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G27" s="9"/>
       <c r="H27" s="10">
@@ -1474,7 +1468,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28" s="9">
         <v>300</v>
@@ -1487,7 +1481,7 @@
         <v>450</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G28" s="9"/>
       <c r="H28" s="10">
@@ -1504,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -1517,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C31" s="9">
         <v>0</v>
@@ -1525,10 +1519,10 @@
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="G31" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="G31" s="9" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -1536,7 +1530,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C32" s="9">
         <v>380</v>
@@ -1550,10 +1544,10 @@
         <v>350</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H32" s="10">
         <v>46271</v>
@@ -1564,7 +1558,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C33" s="9">
         <v>260</v>
@@ -1578,10 +1572,10 @@
         <v>290</v>
       </c>
       <c r="F33" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G33" s="9" t="s">
         <v>71</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="H33" s="10">
         <v>46271</v>
@@ -1592,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C34" s="9">
         <v>300</v>
@@ -1605,10 +1599,10 @@
         <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G34" s="9" t="s">
         <v>74</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -1616,7 +1610,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C35" s="9">
         <v>150</v>
@@ -1629,10 +1623,10 @@
         <v>187.5</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
@@ -1715,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C39" s="9">
         <v>300</v>
@@ -1728,7 +1722,7 @@
         <v>330</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="10">
@@ -1756,7 +1750,7 @@
         <v>31</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
@@ -1764,7 +1758,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C41" s="9">
         <v>400</v>
@@ -1777,10 +1771,10 @@
         <v>520</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H41" s="10">
         <v>46271</v>
@@ -1807,7 +1801,7 @@
         <v>23</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H42" s="10">
         <v>46273</v>
@@ -1818,7 +1812,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C43" s="9">
         <v>500</v>
@@ -1831,7 +1825,7 @@
         <v>475</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G43" s="9"/>
       <c r="H43" s="10">
@@ -1843,7 +1837,7 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -1869,7 +1863,7 @@
         <v>1200</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G45" s="9"/>
     </row>
@@ -1894,7 +1888,7 @@
         <v>44</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H46" s="10">
         <v>46273</v>
@@ -1905,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C47" s="9">
         <v>600</v>
@@ -1918,10 +1912,10 @@
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -1929,7 +1923,7 @@
         <v>0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C48" s="9">
         <v>300</v>
@@ -1942,10 +1936,10 @@
         <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
@@ -1953,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C49" s="9">
         <v>200</v>
@@ -1966,10 +1960,10 @@
         <v>250</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
@@ -1993,14 +1987,14 @@
         <v>23</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="9"/>
       <c r="B51" s="9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
@@ -2035,7 +2029,7 @@
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="9"/>
       <c r="B53" s="9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
@@ -2048,7 +2042,7 @@
         <v>0</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C54" s="9">
         <v>400</v>
@@ -2061,10 +2055,10 @@
         <v>280</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
@@ -2072,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C55" s="9">
         <v>300</v>
@@ -2085,10 +2079,10 @@
         <v>225</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno 16.9.: Eigner 1000 kg Birnen za 1,15; Armand 200 kg Birnen + 150 kg Zwetschken
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{09AAA927-0DB5-412C-99DF-B3C79C2D51C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C47A436-D14B-4234-825F-F5BA19FA1475}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6275A320-1B5B-448A-9B06-ABC6C702CAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -191,6 +191,15 @@
     <t>Lämmererweg 2 5321 Koppl </t>
   </si>
   <si>
+    <t>Armand, Pfarre Koppl</t>
+  </si>
+  <si>
+    <t>Pfarramt Thalgau</t>
+  </si>
+  <si>
+    <t>(47.8450105, 13.2584452) Übergabe in Koppl bei Peter Fuchs</t>
+  </si>
+  <si>
     <t>Herz Jesu</t>
   </si>
   <si>
@@ -260,7 +269,7 @@
     <t>(47.1513091, 13.7456747) Abholung in Salzburg oder Radstadt möglich – Urlaub 9.–18.9.!</t>
   </si>
   <si>
-    <t>Armand, Pfarre Koppl</t>
+    <t>(47.8450105, 13.2584452)</t>
   </si>
   <si>
     <t>Rainer</t>
@@ -336,15 +345,6 @@
   </si>
   <si>
     <t>(47.2765915, 13.3198029)</t>
-  </si>
-  <si>
-    <t>Pfarramt Thalgau</t>
-  </si>
-  <si>
-    <t>(47.8450105, 13.2584452) Übergabe in Koppl bei Peter Fuchs</t>
-  </si>
-  <si>
-    <t>(47.8450105, 13.2584452)</t>
   </si>
 </sst>
 </file>
@@ -352,9 +352,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
-    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -422,21 +422,21 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -1336,7 +1336,7 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="C23" s="3">
         <v>100</v>
@@ -1349,10 +1349,10 @@
         <v>150</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>101</v>
+        <v>53</v>
       </c>
       <c r="G23" t="s">
-        <v>102</v>
+        <v>54</v>
       </c>
       <c r="H23" s="10">
         <v>46222</v>
@@ -1363,7 +1363,7 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C24" s="3">
         <v>360</v>
@@ -1377,10 +1377,10 @@
         <v>400</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G24" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H24" s="10">
         <v>46222</v>
@@ -1391,7 +1391,7 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C25">
         <v>950</v>
@@ -1404,10 +1404,10 @@
         <v>1425</v>
       </c>
       <c r="F25" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G25" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H25" s="10">
         <v>46233</v>
@@ -1418,7 +1418,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C26" s="9">
         <v>300</v>
@@ -1431,7 +1431,7 @@
         <v>450</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G26" s="9"/>
       <c r="H26" s="10">
@@ -1443,7 +1443,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C27" s="9">
         <v>1000</v>
@@ -1456,7 +1456,7 @@
         <v>1500</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G27" s="9"/>
       <c r="H27" s="10">
@@ -1468,7 +1468,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C28" s="9">
         <v>300</v>
@@ -1481,7 +1481,7 @@
         <v>450</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G28" s="9"/>
       <c r="H28" s="10">
@@ -1498,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -1511,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C31" s="9">
         <v>0</v>
@@ -1519,10 +1519,10 @@
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -1530,7 +1530,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C32" s="9">
         <v>380</v>
@@ -1544,10 +1544,10 @@
         <v>350</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H32" s="10">
         <v>46271</v>
@@ -1558,7 +1558,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C33" s="9">
         <v>260</v>
@@ -1572,10 +1572,10 @@
         <v>290</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H33" s="10">
         <v>46271</v>
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C34" s="9">
         <v>300</v>
@@ -1599,18 +1599,18 @@
         <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="C35" s="9">
         <v>150</v>
@@ -1623,10 +1623,13 @@
         <v>187.5</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>101</v>
+        <v>53</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>103</v>
+        <v>78</v>
+      </c>
+      <c r="H35" s="10">
+        <v>46281</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
@@ -1709,7 +1712,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C39" s="9">
         <v>300</v>
@@ -1722,7 +1725,7 @@
         <v>330</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="10">
@@ -1750,7 +1753,7 @@
         <v>31</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
@@ -1758,7 +1761,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C41" s="9">
         <v>400</v>
@@ -1771,10 +1774,10 @@
         <v>520</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H41" s="10">
         <v>46271</v>
@@ -1801,7 +1804,7 @@
         <v>23</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H42" s="10">
         <v>46273</v>
@@ -1812,7 +1815,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C43" s="9">
         <v>500</v>
@@ -1825,7 +1828,7 @@
         <v>475</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G43" s="9"/>
       <c r="H43" s="10">
@@ -1837,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -1847,7 +1850,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B45" s="9" t="s">
         <v>7</v>
@@ -1856,16 +1859,19 @@
         <v>1000</v>
       </c>
       <c r="D45" s="9">
-        <v>1.2</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E45" s="9">
         <f t="shared" ref="E45:E50" si="2">C45*D45</f>
-        <v>1200</v>
+        <v>1150</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G45" s="9"/>
+      <c r="H45" s="10">
+        <v>46281</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="b">
@@ -1888,7 +1894,7 @@
         <v>44</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H46" s="10">
         <v>46273</v>
@@ -1899,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C47" s="9">
         <v>600</v>
@@ -1912,10 +1918,10 @@
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -1923,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C48" s="9">
         <v>300</v>
@@ -1936,18 +1942,18 @@
         <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="C49" s="9">
         <v>200</v>
@@ -1960,10 +1966,13 @@
         <v>250</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>101</v>
+        <v>53</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>103</v>
+        <v>78</v>
+      </c>
+      <c r="H49" s="10">
+        <v>46281</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
@@ -1987,14 +1996,14 @@
         <v>23</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="9"/>
       <c r="B51" s="9" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
@@ -2029,7 +2038,7 @@
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="9"/>
       <c r="B53" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
@@ -2042,7 +2051,7 @@
         <v>0</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C54" s="9">
         <v>400</v>
@@ -2055,10 +2064,10 @@
         <v>280</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
@@ -2066,7 +2075,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C55" s="9">
         <v>300</v>
@@ -2079,10 +2088,10 @@
         <v>225</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
@@ -2096,7 +2105,7 @@
       <c r="D56" s="3"/>
       <c r="E56" s="8">
         <f>SUM(E2:E55)</f>
-        <v>33447.5</v>
+        <v>33397.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Bayer: jablka 400 kg za 0,60 (domluveno), nove 500 kg Birnen Williams za 1,00
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6275A320-1B5B-448A-9B06-ABC6C702CAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902D01C9-C16A-4D80-BBAB-776A897DFE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="104">
   <si>
     <t>Geliefert</t>
   </si>
@@ -323,19 +323,19 @@
     <t>(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
   </si>
   <si>
+    <t>Gerhard Bayer</t>
+  </si>
+  <si>
+    <t>Dorf 14, 5603 Kleinarl</t>
+  </si>
+  <si>
+    <t>Abholung in Salzburg möglich</t>
+  </si>
+  <si>
     <t>Birnen Packham</t>
   </si>
   <si>
     <t>Äpfel</t>
-  </si>
-  <si>
-    <t>Gerhard Bayer</t>
-  </si>
-  <si>
-    <t>Dorf 14, 5603 Kleinarl</t>
-  </si>
-  <si>
-    <t>Abholung in Salzburg möglich – Preis 0,70 noch nicht fix vereinbart</t>
   </si>
   <si>
     <t>Ferdinand Huber</t>
@@ -784,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1862,7 +1862,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="E45" s="9">
-        <f t="shared" ref="E45:E50" si="2">C45*D45</f>
+        <f t="shared" ref="E45:E51" si="2">C45*D45</f>
         <v>1150</v>
       </c>
       <c r="F45" s="9" t="s">
@@ -2001,117 +2001,137 @@
       <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B51" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="9"/>
-      <c r="G51" s="9"/>
+      <c r="C51" s="9">
+        <v>500</v>
+      </c>
+      <c r="D51" s="9">
+        <v>1</v>
+      </c>
+      <c r="E51" s="9">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>98</v>
+      </c>
       <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A52" s="9"/>
       <c r="B52" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C52" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D52" s="9">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E52" s="9">
-        <f>C52*D52</f>
-        <v>1100</v>
-      </c>
-      <c r="F52" s="9" t="s">
-        <v>29</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
       <c r="G52" s="9"/>
       <c r="H52" s="9"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="9"/>
+      <c r="A53" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B53" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="C53" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D53" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E53" s="9">
+        <f>C53*D53</f>
+        <v>1100</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A54" s="9"/>
       <c r="B54" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="C54" s="9">
-        <v>400</v>
-      </c>
-      <c r="D54" s="9">
-        <v>0.7</v>
-      </c>
-      <c r="E54" s="9">
-        <f>C54*D54</f>
-        <v>280</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="G54" s="9" t="s">
         <v>100</v>
       </c>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C55" s="9">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D55" s="9">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E55" s="9">
         <f>C55*D55</f>
+        <v>240</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A56" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C56" s="9">
+        <v>300</v>
+      </c>
+      <c r="D56" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E56" s="9">
+        <f>C56*D56</f>
         <v>225</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="F56" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="G56" s="9" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A56" t="b">
-        <v>0</v>
-      </c>
-      <c r="C56" s="3">
-        <f>SUM(C2:C55)</f>
-        <v>26150</v>
-      </c>
-      <c r="D56" s="3"/>
-      <c r="E56" s="8">
-        <f>SUM(E2:E55)</f>
-        <v>33397.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="b">
         <v>0</v>
       </c>
+      <c r="C57" s="3">
+        <f>SUM(C2:C56)</f>
+        <v>26650</v>
+      </c>
+      <c r="D57" s="3"/>
+      <c r="E57" s="8">
+        <f>SUM(E2:E56)</f>
+        <v>33857.5</v>
+      </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="b">
@@ -2195,6 +2215,11 @@
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ceny 1,15: Schlick 600 kg Birnen, Lackner 300 kg Zwetschken + 300 kg Birnen
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902D01C9-C16A-4D80-BBAB-776A897DFE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E14F2A0-4CB9-4D6E-88D7-0F264F169463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1592,11 +1592,11 @@
         <v>300</v>
       </c>
       <c r="D34" s="9">
-        <v>1.3</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E34" s="9">
         <f t="shared" si="1"/>
-        <v>390</v>
+        <v>345</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>76</v>
@@ -1911,11 +1911,11 @@
         <v>600</v>
       </c>
       <c r="D47" s="9">
-        <v>1.2</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E47" s="9">
         <f t="shared" si="2"/>
-        <v>720</v>
+        <v>690</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>92</v>
@@ -1935,11 +1935,11 @@
         <v>300</v>
       </c>
       <c r="D48" s="9">
-        <v>1.2</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E48" s="9">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>76</v>
@@ -2130,7 +2130,7 @@
       <c r="D57" s="3"/>
       <c r="E57" s="8">
         <f>SUM(E2:E56)</f>
-        <v>33857.5</v>
+        <v>33767.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Lackner: puvodni ceny (Zwetschken 1,30 = 390, Birnen 1,20 = 360)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E14F2A0-4CB9-4D6E-88D7-0F264F169463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51016A9-BF68-40B5-ACF4-0C98525AADA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1592,11 +1592,11 @@
         <v>300</v>
       </c>
       <c r="D34" s="9">
-        <v>1.1499999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="E34" s="9">
         <f t="shared" si="1"/>
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>76</v>
@@ -1935,11 +1935,11 @@
         <v>300</v>
       </c>
       <c r="D48" s="9">
-        <v>1.1499999999999999</v>
+        <v>1.2</v>
       </c>
       <c r="E48" s="9">
         <f t="shared" si="2"/>
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>76</v>
@@ -2130,7 +2130,7 @@
       <c r="D57" s="3"/>
       <c r="E57" s="8">
         <f>SUM(E2:E56)</f>
-        <v>33767.5</v>
+        <v>33827.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Lackner: nakonec 1,15 za Zwetschken i Birnen
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51016A9-BF68-40B5-ACF4-0C98525AADA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4FB057-D6D8-4DB0-8A97-F3A11F50CB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1592,11 +1592,11 @@
         <v>300</v>
       </c>
       <c r="D34" s="9">
-        <v>1.3</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E34" s="9">
         <f t="shared" si="1"/>
-        <v>390</v>
+        <v>345</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>76</v>
@@ -1935,11 +1935,11 @@
         <v>300</v>
       </c>
       <c r="D48" s="9">
-        <v>1.2</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E48" s="9">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>76</v>
@@ -2130,7 +2130,7 @@
       <c r="D57" s="3"/>
       <c r="E57" s="8">
         <f>SUM(E2:E56)</f>
-        <v>33827.5</v>
+        <v>33767.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Lackner: konecne puvodni ceny (Zwetschken 390, Birnen 360)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4FB057-D6D8-4DB0-8A97-F3A11F50CB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3FFC61-5924-43A4-9061-2ECBDD5B607E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1592,11 +1592,11 @@
         <v>300</v>
       </c>
       <c r="D34" s="9">
-        <v>1.1499999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="E34" s="9">
         <f t="shared" si="1"/>
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>76</v>
@@ -1935,11 +1935,11 @@
         <v>300</v>
       </c>
       <c r="D48" s="9">
-        <v>1.1499999999999999</v>
+        <v>1.2</v>
       </c>
       <c r="E48" s="9">
         <f t="shared" si="2"/>
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>76</v>
@@ -2130,7 +2130,7 @@
       <c r="D57" s="3"/>
       <c r="E57" s="8">
         <f>SUM(E2:E56)</f>
-        <v>33767.5</v>
+        <v>33827.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Schlick: presna adresa Lamm 82, 5584 Zederhaus (overeno na dum)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3FFC61-5924-43A4-9061-2ECBDD5B607E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8182E8D-9106-4D5C-95C6-E5C21DEA035F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -311,7 +311,7 @@
     <t>Christian Schlick</t>
   </si>
   <si>
-    <t>Zederhaus</t>
+    <t>Lamm 82, 5584 Zederhaus</t>
   </si>
   <si>
     <t>Abholung in Salzburg oder Radstadt möglich</t>

</xml_diff>

<commit_message>
Lackner: presna adresa Groebendorf 114 (overeno na dum), Zwetschken 340 kg
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8182E8D-9106-4D5C-95C6-E5C21DEA035F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C6AE23-ADF9-498A-A221-91B7BDFE1FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="102">
   <si>
     <t>Geliefert</t>
   </si>
@@ -263,10 +263,10 @@
     <t>Johann Lackner</t>
   </si>
   <si>
-    <t>5571 Mariapfarr</t>
-  </si>
-  <si>
-    <t>(47.1513091, 13.7456747) Abholung in Salzburg oder Radstadt möglich – Urlaub 9.–18.9.!</t>
+    <t>Gröbendorf 114, 5571 Mariapfarr</t>
+  </si>
+  <si>
+    <t>Abholung in Salzburg oder Radstadt möglich</t>
   </si>
   <si>
     <t>(47.8450105, 13.2584452)</t>
@@ -312,12 +312,6 @@
   </si>
   <si>
     <t>Lamm 82, 5584 Zederhaus</t>
-  </si>
-  <si>
-    <t>Abholung in Salzburg oder Radstadt möglich</t>
-  </si>
-  <si>
-    <t>(47.1513091, 13.7456747) – Urlaub 9.–18.9.!</t>
   </si>
   <si>
     <t>(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
@@ -1589,14 +1583,14 @@
         <v>75</v>
       </c>
       <c r="C34" s="9">
-        <v>300</v>
+        <v>340</v>
       </c>
       <c r="D34" s="9">
         <v>1.3</v>
       </c>
       <c r="E34" s="9">
         <f t="shared" si="1"/>
-        <v>390</v>
+        <v>442</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>76</v>
@@ -1921,7 +1915,7 @@
         <v>92</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -1944,9 +1938,7 @@
       <c r="F48" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="G48" s="9" t="s">
-        <v>94</v>
-      </c>
+      <c r="G48" s="9"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="b">
@@ -1996,7 +1988,7 @@
         <v>23</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H50" s="9"/>
     </row>
@@ -2005,7 +1997,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C51" s="9">
         <v>500</v>
@@ -2018,17 +2010,17 @@
         <v>500</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="9"/>
       <c r="B52" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
@@ -2063,7 +2055,7 @@
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="9"/>
       <c r="B54" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
@@ -2076,7 +2068,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C55" s="9">
         <v>400</v>
@@ -2089,10 +2081,10 @@
         <v>240</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
@@ -2100,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C56" s="9">
         <v>300</v>
@@ -2113,10 +2105,10 @@
         <v>225</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
@@ -2125,12 +2117,12 @@
       </c>
       <c r="C57" s="3">
         <f>SUM(C2:C56)</f>
-        <v>26650</v>
+        <v>26690</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="8">
         <f>SUM(E2:E56)</f>
-        <v>33827.5</v>
+        <v>33879.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno 20.9.: Lackner 340 kg Zwetschken za 440 + 300 kg Birnen, Schlick 608 kg za 700
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C6AE23-ADF9-498A-A221-91B7BDFE1FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D555C306-B844-49B9-A708-7EA291F1479B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="103">
   <si>
     <t>Geliefert</t>
   </si>
@@ -266,7 +266,7 @@
     <t>Gröbendorf 114, 5571 Mariapfarr</t>
   </si>
   <si>
-    <t>Abholung in Salzburg oder Radstadt möglich</t>
+    <t>Abholung in Salzburg oder Radstadt möglich – pauschal 440 €</t>
   </si>
   <si>
     <t>(47.8450105, 13.2584452)</t>
@@ -312,6 +312,9 @@
   </si>
   <si>
     <t>Lamm 82, 5584 Zederhaus</t>
+  </si>
+  <si>
+    <t>Abholung in Salzburg oder Radstadt möglich – pauschal 700 €</t>
   </si>
   <si>
     <t>(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
@@ -1577,7 +1580,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B34" s="9" t="s">
         <v>75</v>
@@ -1586,17 +1589,21 @@
         <v>340</v>
       </c>
       <c r="D34" s="9">
-        <v>1.3</v>
+        <f>440/340</f>
+        <v>1.2941176470588236</v>
       </c>
       <c r="E34" s="9">
         <f t="shared" si="1"/>
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>76</v>
       </c>
       <c r="G34" s="9" t="s">
         <v>77</v>
+      </c>
+      <c r="H34" s="10">
+        <v>46285</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -1896,31 +1903,35 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>91</v>
       </c>
       <c r="C47" s="9">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="D47" s="9">
-        <v>1.1499999999999999</v>
+        <f>700/608</f>
+        <v>1.1513157894736843</v>
       </c>
       <c r="E47" s="9">
         <f t="shared" si="2"/>
-        <v>690</v>
+        <v>700</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>92</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>77</v>
+        <v>93</v>
+      </c>
+      <c r="H47" s="10">
+        <v>46285</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>75</v>
@@ -1939,6 +1950,9 @@
         <v>76</v>
       </c>
       <c r="G48" s="9"/>
+      <c r="H48" s="10">
+        <v>46285</v>
+      </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="b">
@@ -1988,7 +2002,7 @@
         <v>23</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H50" s="9"/>
     </row>
@@ -1997,7 +2011,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C51" s="9">
         <v>500</v>
@@ -2010,17 +2024,17 @@
         <v>500</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="9"/>
       <c r="B52" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
@@ -2055,7 +2069,7 @@
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="9"/>
       <c r="B54" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
@@ -2068,7 +2082,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C55" s="9">
         <v>400</v>
@@ -2081,10 +2095,10 @@
         <v>240</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
@@ -2092,7 +2106,7 @@
         <v>0</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C56" s="9">
         <v>300</v>
@@ -2105,10 +2119,10 @@
         <v>225</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
@@ -2117,12 +2131,12 @@
       </c>
       <c r="C57" s="3">
         <f>SUM(C2:C56)</f>
-        <v>26690</v>
+        <v>26698</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="8">
         <f>SUM(E2:E56)</f>
-        <v>33879.5</v>
+        <v>33887.5</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova objednavka: Ferdinand Huber 200 kg Birnen Williams za 1,10
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D555C306-B844-49B9-A708-7EA291F1479B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28FE8EE-F896-4156-88A0-3353AFA8C9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4180" yWindow="4180" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="103">
   <si>
     <t>Geliefert</t>
   </si>
@@ -329,19 +329,19 @@
     <t>Abholung in Salzburg möglich</t>
   </si>
   <si>
+    <t>Ferdinand Huber</t>
+  </si>
+  <si>
+    <t>Kreuzsalgasse 4, 5603 Kleinarl</t>
+  </si>
+  <si>
+    <t>(47.2765915, 13.3198029)</t>
+  </si>
+  <si>
     <t>Birnen Packham</t>
   </si>
   <si>
     <t>Äpfel</t>
-  </si>
-  <si>
-    <t>Ferdinand Huber</t>
-  </si>
-  <si>
-    <t>Kreuzsalgasse 4, 5603 Kleinarl</t>
-  </si>
-  <si>
-    <t>(47.2765915, 13.3198029)</t>
   </si>
 </sst>
 </file>
@@ -781,7 +781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1863,7 +1863,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="E45" s="9">
-        <f t="shared" ref="E45:E51" si="2">C45*D45</f>
+        <f t="shared" ref="E45:E52" si="2">C45*D45</f>
         <v>1150</v>
       </c>
       <c r="F45" s="9" t="s">
@@ -2032,117 +2032,137 @@
       <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="9"/>
+      <c r="A52" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B52" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="9"/>
+      <c r="C52" s="9">
+        <v>200</v>
+      </c>
+      <c r="D52" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E52" s="9">
+        <f t="shared" si="2"/>
+        <v>220.00000000000003</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>100</v>
+      </c>
       <c r="H52" s="9"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A53" s="9"/>
       <c r="B53" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C53" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D53" s="9">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E53" s="9">
-        <f>C53*D53</f>
-        <v>1100</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>29</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
       <c r="G53" s="9"/>
       <c r="H53" s="9"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="9"/>
+      <c r="A54" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B54" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="C54" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D54" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E54" s="9">
+        <f>C54*D54</f>
+        <v>1100</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A55" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A55" s="9"/>
       <c r="B55" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C55" s="9">
-        <v>400</v>
-      </c>
-      <c r="D55" s="9">
-        <v>0.6</v>
-      </c>
-      <c r="E55" s="9">
-        <f>C55*D55</f>
-        <v>240</v>
-      </c>
-      <c r="F55" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>97</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C56" s="9">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D56" s="9">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E56" s="9">
         <f>C56*D56</f>
+        <v>240</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A57" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C57" s="9">
+        <v>300</v>
+      </c>
+      <c r="D57" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E57" s="9">
+        <f>C57*D57</f>
         <v>225</v>
       </c>
-      <c r="F56" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A57" t="b">
-        <v>0</v>
-      </c>
-      <c r="C57" s="3">
-        <f>SUM(C2:C56)</f>
-        <v>26698</v>
-      </c>
-      <c r="D57" s="3"/>
-      <c r="E57" s="8">
-        <f>SUM(E2:E56)</f>
-        <v>33887.5</v>
+      <c r="F57" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="b">
         <v>0</v>
       </c>
+      <c r="C58" s="3">
+        <f>SUM(C2:C57)</f>
+        <v>26898</v>
+      </c>
+      <c r="D58" s="3"/>
+      <c r="E58" s="8">
+        <f>SUM(E2:E57)</f>
+        <v>34107.5</v>
+      </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="b">
@@ -2226,6 +2246,11 @@
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Lukas Oblasser 350 kg Birnen Williams za 1,20, odber Marktparkplatz Wagrain
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28FE8EE-F896-4156-88A0-3353AFA8C9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F18620A-61C0-43A5-9308-C0072DFAE8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4180" yWindow="4180" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="106">
   <si>
     <t>Geliefert</t>
   </si>
@@ -336,6 +336,15 @@
   </si>
   <si>
     <t>(47.2765915, 13.3198029)</t>
+  </si>
+  <si>
+    <t>Lukas Oblasser</t>
+  </si>
+  <si>
+    <t>Marktparkplatz, 5602 Wagrain</t>
+  </si>
+  <si>
+    <t>(47.333582, 13.295091) Abholung am Marktparkplatz Wagrain – Kunde kommt aus Osttirol</t>
   </si>
   <si>
     <t>Birnen Packham</t>
@@ -781,7 +790,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1863,7 +1872,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="E45" s="9">
-        <f t="shared" ref="E45:E52" si="2">C45*D45</f>
+        <f t="shared" ref="E45:E53" si="2">C45*D45</f>
         <v>1150</v>
       </c>
       <c r="F45" s="9" t="s">
@@ -2057,117 +2066,137 @@
       <c r="H52" s="9"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="9"/>
+      <c r="A53" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B53" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
-      <c r="G53" s="9"/>
+      <c r="C53" s="9">
+        <v>350</v>
+      </c>
+      <c r="D53" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E53" s="9">
+        <f t="shared" si="2"/>
+        <v>420</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>103</v>
+      </c>
       <c r="H53" s="9"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A54" s="9"/>
       <c r="B54" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C54" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D54" s="9">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E54" s="9">
-        <f>C54*D54</f>
-        <v>1100</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>29</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
       <c r="G54" s="9"/>
       <c r="H54" s="9"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A55" s="9"/>
+      <c r="A55" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B55" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="C55" s="9"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="C55" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D55" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E55" s="9">
+        <f>C55*D55</f>
+        <v>1100</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A56" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A56" s="9"/>
       <c r="B56" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C56" s="9">
-        <v>400</v>
-      </c>
-      <c r="D56" s="9">
-        <v>0.6</v>
-      </c>
-      <c r="E56" s="9">
-        <f>C56*D56</f>
-        <v>240</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>97</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C57" s="9">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D57" s="9">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E57" s="9">
         <f>C57*D57</f>
+        <v>240</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A58" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C58" s="9">
+        <v>300</v>
+      </c>
+      <c r="D58" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E58" s="9">
+        <f>C58*D58</f>
         <v>225</v>
       </c>
-      <c r="F57" s="9" t="s">
+      <c r="F58" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G58" s="9" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A58" t="b">
-        <v>0</v>
-      </c>
-      <c r="C58" s="3">
-        <f>SUM(C2:C57)</f>
-        <v>26898</v>
-      </c>
-      <c r="D58" s="3"/>
-      <c r="E58" s="8">
-        <f>SUM(E2:E57)</f>
-        <v>34107.5</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="b">
         <v>0</v>
       </c>
+      <c r="C59" s="3">
+        <f>SUM(C2:C58)</f>
+        <v>27248</v>
+      </c>
+      <c r="D59" s="3"/>
+      <c r="E59" s="8">
+        <f>SUM(E2:E58)</f>
+        <v>34527.5</v>
+      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="b">
@@ -2251,6 +2280,11 @@
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Doruceno 22.9.: Oblasser 300 kg, Bayer 400 kg Birnen + 400 kg Apfel, Huber 200+300 kg (vc. 25 EUR dysko)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F18620A-61C0-43A5-9308-C0072DFAE8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1FF1ED-FE9D-45FD-84BF-8B9CBAA95F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="107">
   <si>
     <t>Geliefert</t>
   </si>
@@ -335,22 +335,25 @@
     <t>Kreuzsalgasse 4, 5603 Kleinarl</t>
   </si>
   <si>
+    <t>(47.2765915, 13.3198029) – inkl. 25 € Trinkgeld</t>
+  </si>
+  <si>
+    <t>Lukas Oblasser</t>
+  </si>
+  <si>
+    <t>Marktparkplatz, 5602 Wagrain</t>
+  </si>
+  <si>
+    <t>(47.333582, 13.295091) Abholung am Marktparkplatz Wagrain – Kunde kommt aus Osttirol</t>
+  </si>
+  <si>
+    <t>Birnen Packham</t>
+  </si>
+  <si>
+    <t>Äpfel</t>
+  </si>
+  <si>
     <t>(47.2765915, 13.3198029)</t>
-  </si>
-  <si>
-    <t>Lukas Oblasser</t>
-  </si>
-  <si>
-    <t>Marktparkplatz, 5602 Wagrain</t>
-  </si>
-  <si>
-    <t>(47.333582, 13.295091) Abholung am Marktparkplatz Wagrain – Kunde kommt aus Osttirol</t>
-  </si>
-  <si>
-    <t>Birnen Packham</t>
-  </si>
-  <si>
-    <t>Äpfel</t>
   </si>
 </sst>
 </file>
@@ -1872,7 +1875,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="E45" s="9">
-        <f t="shared" ref="E45:E53" si="2">C45*D45</f>
+        <f t="shared" ref="E45:E51" si="2">C45*D45</f>
         <v>1150</v>
       </c>
       <c r="F45" s="9" t="s">
@@ -2017,20 +2020,20 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>95</v>
       </c>
       <c r="C51" s="9">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="D51" s="9">
         <v>1</v>
       </c>
       <c r="E51" s="9">
         <f t="shared" si="2"/>
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>96</v>
@@ -2038,11 +2041,13 @@
       <c r="G51" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H51" s="9"/>
+      <c r="H51" s="10">
+        <v>46287</v>
+      </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>98</v>
@@ -2054,8 +2059,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="E52" s="9">
-        <f t="shared" si="2"/>
-        <v>220.00000000000003</v>
+        <v>245</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>99</v>
@@ -2063,24 +2067,26 @@
       <c r="G52" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="H52" s="9"/>
+      <c r="H52" s="10">
+        <v>46287</v>
+      </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>101</v>
       </c>
       <c r="C53" s="9">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="D53" s="9">
         <v>1.2</v>
       </c>
       <c r="E53" s="9">
-        <f t="shared" si="2"/>
-        <v>420</v>
+        <f>C53*D53</f>
+        <v>360</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>102</v>
@@ -2088,7 +2094,9 @@
       <c r="G53" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H53" s="9"/>
+      <c r="H53" s="10">
+        <v>46287</v>
+      </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="9"/>
@@ -2138,7 +2146,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" s="9" t="s">
         <v>95</v>
@@ -2159,10 +2167,13 @@
       <c r="G57" s="9" t="s">
         <v>97</v>
       </c>
+      <c r="H57" s="10">
+        <v>46287</v>
+      </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" s="9" t="s">
         <v>98</v>
@@ -2181,7 +2192,10 @@
         <v>99</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
+      </c>
+      <c r="H58" s="10">
+        <v>46287</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
@@ -2190,12 +2204,12 @@
       </c>
       <c r="C59" s="3">
         <f>SUM(C2:C58)</f>
-        <v>27248</v>
+        <v>27098</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="8">
         <f>SUM(E2:E58)</f>
-        <v>34527.5</v>
+        <v>34392.5</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno 29.9.: Moser 1500 kg Zwetschken za 1650 EUR
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1FF1ED-FE9D-45FD-84BF-8B9CBAA95F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3950FA4B-A653-4228-82E9-8D29E34ECAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37300" yWindow="1100" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1747,7 +1747,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B40" s="9" t="s">
         <v>30</v>
@@ -1767,6 +1767,9 @@
       </c>
       <c r="G40" s="9" t="s">
         <v>81</v>
+      </c>
+      <c r="H40" s="10">
+        <v>46294</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova odruda Birnen Alexander Lucas: Moser 1000 kg za 0,80, vlastni barva #a87428
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3950FA4B-A653-4228-82E9-8D29E34ECAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA20F735-BBF6-42CD-9DD9-631BCD95A8CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37300" yWindow="1100" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="108">
   <si>
     <t>Geliefert</t>
   </si>
@@ -348,6 +348,9 @@
   </si>
   <si>
     <t>Birnen Packham</t>
+  </si>
+  <si>
+    <t>Birnen Alexander Lucas</t>
   </si>
   <si>
     <t>Äpfel</t>
@@ -793,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -2146,84 +2149,109 @@
       <c r="E56" s="9"/>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>95</v>
+        <v>30</v>
       </c>
       <c r="C57" s="9">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="D57" s="9">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E57" s="9">
         <f>C57*D57</f>
+        <v>800</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G57" s="9"/>
+      <c r="H57" s="9"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A58" s="9"/>
+      <c r="B58" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="9"/>
+      <c r="G58" s="9"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A59" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C59" s="9">
+        <v>400</v>
+      </c>
+      <c r="D59" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="E59" s="9">
+        <f>C59*D59</f>
         <v>240</v>
       </c>
-      <c r="F57" s="9" t="s">
+      <c r="F59" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G59" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H57" s="10">
+      <c r="H59" s="10">
         <v>46287</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A58" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B58" s="9" t="s">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A60" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B60" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C60" s="9">
         <v>300</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D60" s="9">
         <v>0.75</v>
       </c>
-      <c r="E58" s="9">
-        <f>C58*D58</f>
+      <c r="E60" s="9">
+        <f>C60*D60</f>
         <v>225</v>
       </c>
-      <c r="F58" s="9" t="s">
+      <c r="F60" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="G58" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="H58" s="10">
+      <c r="G60" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H60" s="10">
         <v>46287</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A59" t="b">
-        <v>0</v>
-      </c>
-      <c r="C59" s="3">
-        <f>SUM(C2:C58)</f>
-        <v>27098</v>
-      </c>
-      <c r="D59" s="3"/>
-      <c r="E59" s="8">
-        <f>SUM(E2:E58)</f>
-        <v>34392.5</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A60" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="b">
         <v>0</v>
       </c>
+      <c r="C61" s="3">
+        <f>SUM(C2:C60)</f>
+        <v>28098</v>
+      </c>
+      <c r="D61" s="3"/>
+      <c r="E61" s="8">
+        <f>SUM(E2:E60)</f>
+        <v>35192.5</v>
+      </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="b">
@@ -2302,6 +2330,16 @@
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Alexander Lucas svetle zelena; nova odruda Konference (Gasteiger 1000 kg za 0,90); Gasteiger adresa s Bad Ischl
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA20F735-BBF6-42CD-9DD9-631BCD95A8CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFE398B-3165-4B5B-8616-D5050CEF1DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37300" yWindow="1100" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="109">
   <si>
     <t>Geliefert</t>
   </si>
@@ -167,7 +167,7 @@
     <t>Gasteiger</t>
   </si>
   <si>
-    <t>Auweg 73, 4820</t>
+    <t>Auweg 73, 4820 Bad Ischl</t>
   </si>
   <si>
     <t>1 Großkiste</t>
@@ -351,6 +351,9 @@
   </si>
   <si>
     <t>Birnen Alexander Lucas</t>
+  </si>
+  <si>
+    <t>Birnen Konference</t>
   </si>
   <si>
     <t>Äpfel</t>
@@ -796,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -2184,84 +2187,109 @@
       <c r="E58" s="9"/>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>95</v>
+        <v>43</v>
       </c>
       <c r="C59" s="9">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="D59" s="9">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="E59" s="9">
         <f>C59*D59</f>
+        <v>900</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A60" s="9"/>
+      <c r="B60" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A61" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C61" s="9">
+        <v>400</v>
+      </c>
+      <c r="D61" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="E61" s="9">
+        <f>C61*D61</f>
         <v>240</v>
       </c>
-      <c r="F59" s="9" t="s">
+      <c r="F61" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="G59" s="9" t="s">
+      <c r="G61" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H59" s="10">
+      <c r="H61" s="10">
         <v>46287</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A60" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B60" s="9" t="s">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A62" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B62" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="C60" s="9">
+      <c r="C62" s="9">
         <v>300</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D62" s="9">
         <v>0.75</v>
       </c>
-      <c r="E60" s="9">
-        <f>C60*D60</f>
+      <c r="E62" s="9">
+        <f>C62*D62</f>
         <v>225</v>
       </c>
-      <c r="F60" s="9" t="s">
+      <c r="F62" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="G60" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="H60" s="10">
+      <c r="G62" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H62" s="10">
         <v>46287</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A61" t="b">
-        <v>0</v>
-      </c>
-      <c r="C61" s="3">
-        <f>SUM(C2:C60)</f>
-        <v>28098</v>
-      </c>
-      <c r="D61" s="3"/>
-      <c r="E61" s="8">
-        <f>SUM(E2:E60)</f>
-        <v>35192.5</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A62" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="b">
         <v>0</v>
       </c>
+      <c r="C63" s="3">
+        <f>SUM(C2:C62)</f>
+        <v>29098</v>
+      </c>
+      <c r="D63" s="3"/>
+      <c r="E63" s="8">
+        <f>SUM(E2:E62)</f>
+        <v>36092.5</v>
+      </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="b">
@@ -2340,6 +2368,16 @@
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Gasteiger: 500 kg Alexander Lucas + 500 kg Konference (misto 1000), dovoz nejradeji so 3.10. vecer
Cena Lucas zatim chybi (Preis ergänzen). TRUE/FALSE ve sloupci A zase jako hodnoty (LibreOffice je minule ulozil jako vzorce).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="115">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -340,7 +340,13 @@
     <t xml:space="preserve">Birnen Alexander Lucas</t>
   </si>
   <si>
+    <t xml:space="preserve">Preis ergänzen – Lieferung am liebsten Sa 3.10. abends</t>
+  </si>
+  <si>
     <t xml:space="preserve">Birnen Konference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -365,13 +371,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="0&quot; kg&quot;"/>
-    <numFmt numFmtId="167" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_-&quot;€ &quot;* #,##0.00_-;&quot;-€ &quot;* #,##0.00_-;_-&quot;€ &quot;* \-??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;€ &quot;* #,##0.00_-;&quot;-€ &quot;* #,##0.00_-;_-&quot;€ &quot;* \-??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -450,7 +455,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -471,19 +476,60 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  </cellStyleXfs>
+  <cellXfs count="15">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -491,59 +537,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -797,34 +802,33 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="n">
@@ -837,20 +841,19 @@
         <f aca="false">C2*D2</f>
         <v>900</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="2"/>
       <c r="H2" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
@@ -862,20 +865,19 @@
       <c r="E3" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="1"/>
+      <c r="G3" s="2"/>
       <c r="H3" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
@@ -888,20 +890,19 @@
         <f aca="false">C4*D4</f>
         <v>1500</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="1"/>
+      <c r="G4" s="2"/>
       <c r="H4" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="3" t="n">
@@ -913,22 +914,21 @@
       <c r="E5" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H5" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="3" t="n">
@@ -941,20 +941,19 @@
         <f aca="false">C6*D6</f>
         <v>525</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="1"/>
+      <c r="G6" s="2"/>
       <c r="H6" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="3" t="n">
@@ -967,22 +966,21 @@
         <f aca="false">C7*D7</f>
         <v>1500</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="3" t="n">
@@ -998,19 +996,18 @@
       <c r="F8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>46238</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="3" t="n">
@@ -1026,17 +1023,16 @@
       <c r="F9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="2"/>
       <c r="H9" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="3" t="n">
@@ -1052,19 +1048,18 @@
       <c r="F10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="3" t="n">
@@ -1076,22 +1071,21 @@
       <c r="E11" s="4" t="n">
         <v>170</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="3" t="n">
@@ -1104,20 +1098,19 @@
         <f aca="false">C12*D12</f>
         <v>960</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="1"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="3" t="n">
@@ -1133,17 +1126,16 @@
       <c r="F13" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="1"/>
+      <c r="G13" s="2"/>
       <c r="H13" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C14" s="3" t="n">
@@ -1156,20 +1148,19 @@
         <f aca="false">C14*D14</f>
         <v>1000</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="1"/>
+      <c r="G14" s="2"/>
       <c r="H14" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C15" s="3" t="n">
@@ -1182,20 +1173,19 @@
         <f aca="false">C15*D15</f>
         <v>90</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="1"/>
+      <c r="G15" s="2"/>
       <c r="H15" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="3" t="n">
@@ -1208,22 +1198,21 @@
         <f aca="false">C16*D16</f>
         <v>225</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" s="2" t="s">
         <v>37</v>
       </c>
       <c r="H16" s="5" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C17" s="3" t="n">
@@ -1236,20 +1225,19 @@
         <f aca="false">C17*D17</f>
         <v>840</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="1"/>
+      <c r="G17" s="2"/>
       <c r="H17" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C18" s="3" t="n">
@@ -1265,19 +1253,18 @@
       <c r="F18" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="2" t="s">
         <v>42</v>
       </c>
       <c r="H18" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C19" s="3" t="n">
@@ -1290,22 +1277,21 @@
         <f aca="false">C19*D19</f>
         <v>750</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="2" t="s">
         <v>45</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B20" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="3" t="n">
@@ -1321,17 +1307,16 @@
       <c r="F20" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G20" s="1"/>
+      <c r="G20" s="2"/>
       <c r="H20" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>48</v>
       </c>
       <c r="C21" s="3" t="n">
@@ -1347,17 +1332,16 @@
       <c r="F21" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G21" s="1"/>
+      <c r="G21" s="2"/>
       <c r="H21" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>50</v>
       </c>
       <c r="C22" s="3" t="n">
@@ -1373,17 +1357,16 @@
       <c r="F22" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="G22" s="1"/>
+      <c r="G22" s="2"/>
       <c r="H22" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B23" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C23" s="3" t="n">
@@ -1399,19 +1382,18 @@
       <c r="F23" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="G23" s="2" t="s">
         <v>54</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C24" s="3" t="n">
@@ -1428,283 +1410,271 @@
       <c r="F24" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="G24" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H24" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B25" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>950</v>
       </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <f aca="false">C25*D25</f>
         <v>1425</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="G25" s="2" t="s">
         <v>60</v>
       </c>
       <c r="H25" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B26" s="1" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <f aca="false">C26*D26</f>
         <v>450</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="1"/>
+      <c r="G26" s="2"/>
       <c r="H26" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B27" s="1" t="s">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="D27" s="1" t="n">
+      <c r="D27" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <f aca="false">C27*D27</f>
         <v>1500</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G27" s="1"/>
+      <c r="G27" s="2"/>
       <c r="H27" s="5" t="n">
         <v>46238</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B28" s="1" t="s">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <f aca="false">C28*D28</f>
         <v>450</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G28" s="1"/>
+      <c r="G28" s="2"/>
       <c r="H28" s="5" t="n">
         <v>46238</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B30" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-    </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1" t="s">
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="G31" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B32" s="1" t="s">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="2" t="n">
         <v>380</v>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="2" t="n">
         <f aca="false">350/380</f>
         <v>0.921052631578947</v>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="2" t="n">
         <f aca="false">C32*D32</f>
         <v>350</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="G32" s="2" t="s">
         <v>71</v>
       </c>
       <c r="H32" s="5" t="n">
         <v>46271</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B33" s="1" t="s">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="2" t="n">
         <v>260</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="2" t="n">
         <f aca="false">290/260</f>
         <v>1.11538461538462</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <f aca="false">C33*D33</f>
         <v>290</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="G33" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>46271</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B34" s="1" t="s">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="2" t="n">
         <v>340</v>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="2" t="n">
         <f aca="false">440/340</f>
         <v>1.29411764705882</v>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="2" t="n">
         <f aca="false">C34*D34</f>
         <v>440</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G34" s="1" t="s">
+      <c r="G34" s="2" t="s">
         <v>77</v>
       </c>
       <c r="H34" s="5" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B35" s="1" t="s">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D35" s="1" t="n">
+      <c r="D35" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="2" t="n">
         <f aca="false">C35*D35</f>
         <v>187.5</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="G35" s="2" t="s">
         <v>78</v>
       </c>
       <c r="H35" s="5" t="n">
         <v>46281</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -1728,9 +1698,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -1754,9 +1723,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -1780,9 +1748,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -1806,9 +1773,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -1834,9 +1800,8 @@
         <v>46294</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -1862,9 +1827,8 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -1890,9 +1854,8 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -1916,23 +1879,17 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -1956,9 +1913,8 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -1984,9 +1940,8 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -2013,9 +1968,8 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -2039,9 +1993,8 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -2067,9 +2020,8 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -2091,11 +2043,9 @@
       <c r="G50" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H50" s="1"/>
-    </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -2121,9 +2071,8 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B52" s="1" t="s">
@@ -2148,9 +2097,8 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B53" s="1" t="s">
@@ -2176,21 +2124,15 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1"/>
       <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
       <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
-    </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
@@ -2210,23 +2152,16 @@
         <v>29</v>
       </c>
       <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-    </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1"/>
       <c r="B56" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
       <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
@@ -2246,262 +2181,252 @@
         <v>31</v>
       </c>
       <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="E58" s="1" t="n">
+        <f aca="false">C58*D58</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G58" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C58" s="1"/>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
-    </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="11" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
+      <c r="H58" s="14"/>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G59" s="1"/>
+    </row>
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C59" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D59" s="1" t="n">
+      <c r="C60" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="D60" s="1" t="n">
         <v>0.9</v>
       </c>
-      <c r="E59" s="1" t="n">
-        <f aca="false">C59*D59</f>
-        <v>900</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="E60" s="1" t="n">
+        <f aca="false">C60*D60</f>
+        <v>450</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-    </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="0" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B61" s="0" t="s">
+      <c r="G60" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C61" s="0" t="n">
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B61" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D61" s="0" t="n">
+      <c r="D62" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E61" s="0" t="n">
-        <f aca="false">C61*D61</f>
+      <c r="E62" s="1" t="n">
+        <f aca="false">C62*D62</f>
         <v>320</v>
       </c>
-      <c r="F61" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="G61" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="H61" s="5"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1" t="s">
+      <c r="F62" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C62" s="1"/>
-      <c r="D62" s="1"/>
-      <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
+      <c r="G62" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G63" s="1"/>
+    </row>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C63" s="1" t="n">
+      <c r="C64" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D63" s="1" t="n">
+      <c r="D64" s="1" t="n">
         <v>0.6</v>
-      </c>
-      <c r="E63" s="1" t="n">
-        <f aca="false">C63*D63</f>
-        <v>240</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H63" s="5" t="n">
-        <v>46287</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="D64" s="1" t="n">
-        <v>0.75</v>
       </c>
       <c r="E64" s="1" t="n">
         <f aca="false">C64*D64</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>46287</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="C65" s="3" t="n">
-        <f aca="false">SUM(C2:C64)</f>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D65" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E65" s="1" t="n">
+        <f aca="false">C65*D65</f>
+        <v>225</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>46287</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <f aca="false">SUM(C2:C65)</f>
         <v>29498</v>
       </c>
-      <c r="D65" s="3"/>
-      <c r="E65" s="12" t="n">
-        <f aca="false">SUM(E2:E64)</f>
-        <v>36412.5</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2" t="b">
-        <f aca="false">FALSE()</f>
+      <c r="D66" s="3"/>
+      <c r="E66" s="4" t="n">
+        <f aca="false">SUM(E2:E65)</f>
+        <v>35962.5</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Gasteiger: 500 kg Alexander Lucas + 500 kg Konference, so 3. 10. večer (#5)
Cena Lucas zatim chybi (Preis ergänzen). TRUE/FALSE ve sloupci A zase jako hodnoty (LibreOffice je minule ulozil jako vzorce).


Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="115">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -340,7 +340,13 @@
     <t xml:space="preserve">Birnen Alexander Lucas</t>
   </si>
   <si>
+    <t xml:space="preserve">Preis ergänzen – Lieferung am liebsten Sa 3.10. abends</t>
+  </si>
+  <si>
     <t xml:space="preserve">Birnen Konference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -365,13 +371,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="0&quot; kg&quot;"/>
-    <numFmt numFmtId="167" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_-&quot;€ &quot;* #,##0.00_-;&quot;-€ &quot;* #,##0.00_-;_-&quot;€ &quot;* \-??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;€ &quot;* #,##0.00_-;&quot;-€ &quot;* #,##0.00_-;_-&quot;€ &quot;* \-??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -450,7 +455,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -471,19 +476,60 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  </cellStyleXfs>
+  <cellXfs count="15">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -491,59 +537,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -797,34 +802,33 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="n">
@@ -837,20 +841,19 @@
         <f aca="false">C2*D2</f>
         <v>900</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="2"/>
       <c r="H2" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
@@ -862,20 +865,19 @@
       <c r="E3" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="1"/>
+      <c r="G3" s="2"/>
       <c r="H3" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
@@ -888,20 +890,19 @@
         <f aca="false">C4*D4</f>
         <v>1500</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="1"/>
+      <c r="G4" s="2"/>
       <c r="H4" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="3" t="n">
@@ -913,22 +914,21 @@
       <c r="E5" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H5" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="3" t="n">
@@ -941,20 +941,19 @@
         <f aca="false">C6*D6</f>
         <v>525</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="1"/>
+      <c r="G6" s="2"/>
       <c r="H6" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="3" t="n">
@@ -967,22 +966,21 @@
         <f aca="false">C7*D7</f>
         <v>1500</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="3" t="n">
@@ -998,19 +996,18 @@
       <c r="F8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>46238</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="3" t="n">
@@ -1026,17 +1023,16 @@
       <c r="F9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="2"/>
       <c r="H9" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="3" t="n">
@@ -1052,19 +1048,18 @@
       <c r="F10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="3" t="n">
@@ -1076,22 +1071,21 @@
       <c r="E11" s="4" t="n">
         <v>170</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="3" t="n">
@@ -1104,20 +1098,19 @@
         <f aca="false">C12*D12</f>
         <v>960</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="1"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="3" t="n">
@@ -1133,17 +1126,16 @@
       <c r="F13" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="1"/>
+      <c r="G13" s="2"/>
       <c r="H13" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C14" s="3" t="n">
@@ -1156,20 +1148,19 @@
         <f aca="false">C14*D14</f>
         <v>1000</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="1"/>
+      <c r="G14" s="2"/>
       <c r="H14" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C15" s="3" t="n">
@@ -1182,20 +1173,19 @@
         <f aca="false">C15*D15</f>
         <v>90</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="1"/>
+      <c r="G15" s="2"/>
       <c r="H15" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="3" t="n">
@@ -1208,22 +1198,21 @@
         <f aca="false">C16*D16</f>
         <v>225</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" s="2" t="s">
         <v>37</v>
       </c>
       <c r="H16" s="5" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C17" s="3" t="n">
@@ -1236,20 +1225,19 @@
         <f aca="false">C17*D17</f>
         <v>840</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="1"/>
+      <c r="G17" s="2"/>
       <c r="H17" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C18" s="3" t="n">
@@ -1265,19 +1253,18 @@
       <c r="F18" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="2" t="s">
         <v>42</v>
       </c>
       <c r="H18" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C19" s="3" t="n">
@@ -1290,22 +1277,21 @@
         <f aca="false">C19*D19</f>
         <v>750</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="2" t="s">
         <v>45</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B20" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="3" t="n">
@@ -1321,17 +1307,16 @@
       <c r="F20" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G20" s="1"/>
+      <c r="G20" s="2"/>
       <c r="H20" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>48</v>
       </c>
       <c r="C21" s="3" t="n">
@@ -1347,17 +1332,16 @@
       <c r="F21" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G21" s="1"/>
+      <c r="G21" s="2"/>
       <c r="H21" s="5" t="n">
         <v>46229</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>50</v>
       </c>
       <c r="C22" s="3" t="n">
@@ -1373,17 +1357,16 @@
       <c r="F22" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="G22" s="1"/>
+      <c r="G22" s="2"/>
       <c r="H22" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B23" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C23" s="3" t="n">
@@ -1399,19 +1382,18 @@
       <c r="F23" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="G23" s="2" t="s">
         <v>54</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C24" s="3" t="n">
@@ -1428,283 +1410,271 @@
       <c r="F24" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="G24" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H24" s="5" t="n">
         <v>46222</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B25" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>950</v>
       </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <f aca="false">C25*D25</f>
         <v>1425</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="G25" s="2" t="s">
         <v>60</v>
       </c>
       <c r="H25" s="5" t="n">
         <v>46233</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B26" s="1" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <f aca="false">C26*D26</f>
         <v>450</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="1"/>
+      <c r="G26" s="2"/>
       <c r="H26" s="5" t="n">
         <v>46231</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B27" s="1" t="s">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="D27" s="1" t="n">
+      <c r="D27" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <f aca="false">C27*D27</f>
         <v>1500</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G27" s="1"/>
+      <c r="G27" s="2"/>
       <c r="H27" s="5" t="n">
         <v>46238</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B28" s="1" t="s">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <f aca="false">C28*D28</f>
         <v>450</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G28" s="1"/>
+      <c r="G28" s="2"/>
       <c r="H28" s="5" t="n">
         <v>46238</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B30" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-    </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1" t="s">
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="G31" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B32" s="1" t="s">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="2" t="n">
         <v>380</v>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="2" t="n">
         <f aca="false">350/380</f>
         <v>0.921052631578947</v>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="2" t="n">
         <f aca="false">C32*D32</f>
         <v>350</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="G32" s="2" t="s">
         <v>71</v>
       </c>
       <c r="H32" s="5" t="n">
         <v>46271</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B33" s="1" t="s">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="2" t="n">
         <v>260</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="2" t="n">
         <f aca="false">290/260</f>
         <v>1.11538461538462</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <f aca="false">C33*D33</f>
         <v>290</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="G33" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>46271</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B34" s="1" t="s">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="2" t="n">
         <v>340</v>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="2" t="n">
         <f aca="false">440/340</f>
         <v>1.29411764705882</v>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="2" t="n">
         <f aca="false">C34*D34</f>
         <v>440</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G34" s="1" t="s">
+      <c r="G34" s="2" t="s">
         <v>77</v>
       </c>
       <c r="H34" s="5" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B35" s="1" t="s">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="D35" s="1" t="n">
+      <c r="D35" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="2" t="n">
         <f aca="false">C35*D35</f>
         <v>187.5</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="G35" s="2" t="s">
         <v>78</v>
       </c>
       <c r="H35" s="5" t="n">
         <v>46281</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -1728,9 +1698,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -1754,9 +1723,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -1780,9 +1748,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -1806,9 +1773,8 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -1834,9 +1800,8 @@
         <v>46294</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -1862,9 +1827,8 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -1890,9 +1854,8 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -1916,23 +1879,17 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -1956,9 +1913,8 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -1984,9 +1940,8 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -2013,9 +1968,8 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -2039,9 +1993,8 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -2067,9 +2020,8 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -2091,11 +2043,9 @@
       <c r="G50" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H50" s="1"/>
-    </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -2121,9 +2071,8 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B52" s="1" t="s">
@@ -2148,9 +2097,8 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="b">
-        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="B53" s="1" t="s">
@@ -2176,21 +2124,15 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1"/>
       <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
       <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
-    </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
@@ -2210,23 +2152,16 @@
         <v>29</v>
       </c>
       <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-    </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1"/>
       <c r="B56" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
       <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="b">
-        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
@@ -2246,262 +2181,252 @@
         <v>31</v>
       </c>
       <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="E58" s="1" t="n">
+        <f aca="false">C58*D58</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G58" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C58" s="1"/>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
-    </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="11" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
+      <c r="H58" s="14"/>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G59" s="1"/>
+    </row>
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C59" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D59" s="1" t="n">
+      <c r="C60" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="D60" s="1" t="n">
         <v>0.9</v>
       </c>
-      <c r="E59" s="1" t="n">
-        <f aca="false">C59*D59</f>
-        <v>900</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="E60" s="1" t="n">
+        <f aca="false">C60*D60</f>
+        <v>450</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-    </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="0" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B61" s="0" t="s">
+      <c r="G60" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C61" s="0" t="n">
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B61" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D61" s="0" t="n">
+      <c r="D62" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E61" s="0" t="n">
-        <f aca="false">C61*D61</f>
+      <c r="E62" s="1" t="n">
+        <f aca="false">C62*D62</f>
         <v>320</v>
       </c>
-      <c r="F61" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="G61" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="H61" s="5"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1" t="s">
+      <c r="F62" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C62" s="1"/>
-      <c r="D62" s="1"/>
-      <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
+      <c r="G62" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G63" s="1"/>
+    </row>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C63" s="1" t="n">
+      <c r="C64" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D63" s="1" t="n">
+      <c r="D64" s="1" t="n">
         <v>0.6</v>
-      </c>
-      <c r="E63" s="1" t="n">
-        <f aca="false">C63*D63</f>
-        <v>240</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H63" s="5" t="n">
-        <v>46287</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="11" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="D64" s="1" t="n">
-        <v>0.75</v>
       </c>
       <c r="E64" s="1" t="n">
         <f aca="false">C64*D64</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>46287</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="C65" s="3" t="n">
-        <f aca="false">SUM(C2:C64)</f>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D65" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E65" s="1" t="n">
+        <f aca="false">C65*D65</f>
+        <v>225</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>46287</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <f aca="false">SUM(C2:C65)</f>
         <v>29498</v>
       </c>
-      <c r="D65" s="3"/>
-      <c r="E65" s="12" t="n">
-        <f aca="false">SUM(E2:E64)</f>
-        <v>36412.5</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2" t="b">
-        <f aca="false">FALSE()</f>
+      <c r="D66" s="3"/>
+      <c r="E66" s="4" t="n">
+        <f aca="false">SUM(E2:E65)</f>
+        <v>35962.5</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Gasteiger: Konference i Alexander Lucas za 0,95 EUR/kg (2x 475 EUR)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="114">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -340,13 +340,10 @@
     <t xml:space="preserve">Birnen Alexander Lucas</t>
   </si>
   <si>
-    <t xml:space="preserve">Preis ergänzen – Lieferung am liebsten Sa 3.10. abends</t>
+    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -480,7 +477,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,18 +523,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2183,7 +2168,7 @@
       <c r="G57" s="1"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="b">
+      <c r="A58" s="11" t="b">
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -2192,17 +2177,20 @@
       <c r="C58" s="1" t="n">
         <v>500</v>
       </c>
+      <c r="D58" s="1" t="n">
+        <v>0.95</v>
+      </c>
       <c r="E58" s="1" t="n">
         <f aca="false">C58*D58</f>
-        <v>0</v>
+        <v>475</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G58" s="13" t="s">
+      <c r="G58" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="14"/>
+      <c r="H58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1"/>
@@ -2222,22 +2210,22 @@
         <v>500</v>
       </c>
       <c r="D60" s="1" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E60" s="1" t="n">
         <f aca="false">C60*D60</f>
-        <v>450</v>
+        <v>475</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>44</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2245,7 +2233,7 @@
         <v>0</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C62" s="1" t="n">
         <v>400</v>
@@ -2258,17 +2246,17 @@
         <v>320</v>
       </c>
       <c r="F62" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="H62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G63" s="1"/>
     </row>
@@ -2320,7 +2308,7 @@
         <v>99</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H65" s="5" t="n">
         <v>46287</v>
@@ -2337,7 +2325,7 @@
       <c r="D66" s="3"/>
       <c r="E66" s="4" t="n">
         <f aca="false">SUM(E2:E65)</f>
-        <v>35962.5</v>
+        <v>36462.5</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2425,7 +2413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Gasteiger: Konference i Alexander Lucas za 0,95 €/kg (#6)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="114">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -340,13 +340,10 @@
     <t xml:space="preserve">Birnen Alexander Lucas</t>
   </si>
   <si>
-    <t xml:space="preserve">Preis ergänzen – Lieferung am liebsten Sa 3.10. abends</t>
+    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -480,7 +477,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,18 +523,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2183,7 +2168,7 @@
       <c r="G57" s="1"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="b">
+      <c r="A58" s="11" t="b">
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -2192,17 +2177,20 @@
       <c r="C58" s="1" t="n">
         <v>500</v>
       </c>
+      <c r="D58" s="1" t="n">
+        <v>0.95</v>
+      </c>
       <c r="E58" s="1" t="n">
         <f aca="false">C58*D58</f>
-        <v>0</v>
+        <v>475</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G58" s="13" t="s">
+      <c r="G58" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="14"/>
+      <c r="H58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1"/>
@@ -2222,22 +2210,22 @@
         <v>500</v>
       </c>
       <c r="D60" s="1" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E60" s="1" t="n">
         <f aca="false">C60*D60</f>
-        <v>450</v>
+        <v>475</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>44</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2245,7 +2233,7 @@
         <v>0</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C62" s="1" t="n">
         <v>400</v>
@@ -2258,17 +2246,17 @@
         <v>320</v>
       </c>
       <c r="F62" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="H62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G63" s="1"/>
     </row>
@@ -2320,7 +2308,7 @@
         <v>99</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H65" s="5" t="n">
         <v>46287</v>
@@ -2337,7 +2325,7 @@
       <c r="D66" s="3"/>
       <c r="E66" s="4" t="n">
         <f aca="false">SUM(E2:E65)</f>
-        <v>35962.5</v>
+        <v>36462.5</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2425,7 +2413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Kadar: Williams 400 kg za 1,20 + Alexander Lucas/Konference za 0,90 (mnozstvi zatim nezname); doma az od ne 4.10. v poledne, vylozit lze i bez nej
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="115">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -304,7 +304,7 @@
     <t xml:space="preserve">Abholung in Salzburg oder Radstadt möglich – pauschal 700 €</t>
   </si>
   <si>
-    <t xml:space="preserve">(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
+    <t xml:space="preserve">(47.6422225, 13.7605517) Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
   </si>
   <si>
     <t xml:space="preserve">Gerhard Bayer</t>
@@ -341,6 +341,9 @@
   </si>
   <si>
     <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(47.6422225, 13.7605517) oder Konference (egal) – Menge noch offen – Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
@@ -477,7 +480,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,6 +526,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,7 +802,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2193,122 +2208,117 @@
       <c r="H58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1"/>
+      <c r="A59" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B59" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <f aca="false">C59*D59</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G59" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="G59" s="1"/>
+      <c r="H59" s="14"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="11" t="b">
-        <v>0</v>
-      </c>
+      <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G60" s="1"/>
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C60" s="1" t="n">
+      <c r="C61" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="D60" s="1" t="n">
+      <c r="D61" s="1" t="n">
         <v>0.95</v>
       </c>
-      <c r="E60" s="1" t="n">
-        <f aca="false">C60*D60</f>
+      <c r="E61" s="1" t="n">
+        <f aca="false">C61*D61</f>
         <v>475</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B62" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C62" s="1" t="n">
+    </row>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C63" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D62" s="1" t="n">
+      <c r="D63" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E62" s="1" t="n">
-        <f aca="false">C62*D62</f>
+      <c r="E63" s="1" t="n">
+        <f aca="false">C63*D63</f>
         <v>320</v>
       </c>
-      <c r="F62" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G62" s="1" t="s">
+      <c r="F63" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="G63" s="1"/>
+      <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D64" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E64" s="1" t="n">
-        <f aca="false">C64*D64</f>
-        <v>240</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H64" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="G64" s="1"/>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C65" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E65" s="1" t="n">
         <f aca="false">C65*D65</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="H65" s="5" t="n">
         <v>46287</v>
@@ -2316,22 +2326,44 @@
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C66" s="3" t="n">
-        <f aca="false">SUM(C2:C65)</f>
-        <v>29498</v>
-      </c>
-      <c r="D66" s="3"/>
-      <c r="E66" s="4" t="n">
-        <f aca="false">SUM(E2:E65)</f>
-        <v>36462.5</v>
+        <v>1</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E66" s="1" t="n">
+        <f aca="false">C66*D66</f>
+        <v>225</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H66" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C67" s="3" t="n">
+        <f aca="false">SUM(C2:C66)</f>
+        <v>29498</v>
+      </c>
+      <c r="D67" s="3"/>
+      <c r="E67" s="4" t="n">
+        <f aca="false">SUM(E2:E66)</f>
+        <v>36462.5</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
@@ -2415,6 +2447,11 @@
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Kadar: Williams 400 kg + Lucas/Konference za 0,90, od ne 4. 10. (#7)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="115">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -304,7 +304,7 @@
     <t xml:space="preserve">Abholung in Salzburg oder Radstadt möglich – pauschal 700 €</t>
   </si>
   <si>
-    <t xml:space="preserve">(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
+    <t xml:space="preserve">(47.6422225, 13.7605517) Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
   </si>
   <si>
     <t xml:space="preserve">Gerhard Bayer</t>
@@ -341,6 +341,9 @@
   </si>
   <si>
     <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(47.6422225, 13.7605517) oder Konference (egal) – Menge noch offen – Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
@@ -477,7 +480,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,6 +526,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,7 +802,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2193,122 +2208,117 @@
       <c r="H58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1"/>
+      <c r="A59" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B59" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <f aca="false">C59*D59</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G59" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="G59" s="1"/>
+      <c r="H59" s="14"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="11" t="b">
-        <v>0</v>
-      </c>
+      <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G60" s="1"/>
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C60" s="1" t="n">
+      <c r="C61" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="D60" s="1" t="n">
+      <c r="D61" s="1" t="n">
         <v>0.95</v>
       </c>
-      <c r="E60" s="1" t="n">
-        <f aca="false">C60*D60</f>
+      <c r="E61" s="1" t="n">
+        <f aca="false">C61*D61</f>
         <v>475</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B62" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C62" s="1" t="n">
+    </row>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C63" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D62" s="1" t="n">
+      <c r="D63" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E62" s="1" t="n">
-        <f aca="false">C62*D62</f>
+      <c r="E63" s="1" t="n">
+        <f aca="false">C63*D63</f>
         <v>320</v>
       </c>
-      <c r="F62" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G62" s="1" t="s">
+      <c r="F63" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="G63" s="1"/>
+      <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D64" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E64" s="1" t="n">
-        <f aca="false">C64*D64</f>
-        <v>240</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H64" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="G64" s="1"/>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C65" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E65" s="1" t="n">
         <f aca="false">C65*D65</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="H65" s="5" t="n">
         <v>46287</v>
@@ -2316,22 +2326,44 @@
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C66" s="3" t="n">
-        <f aca="false">SUM(C2:C65)</f>
-        <v>29498</v>
-      </c>
-      <c r="D66" s="3"/>
-      <c r="E66" s="4" t="n">
-        <f aca="false">SUM(E2:E65)</f>
-        <v>36462.5</v>
+        <v>1</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E66" s="1" t="n">
+        <f aca="false">C66*D66</f>
+        <v>225</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H66" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C67" s="3" t="n">
+        <f aca="false">SUM(C2:C66)</f>
+        <v>29498</v>
+      </c>
+      <c r="D67" s="3"/>
+      <c r="E67" s="4" t="n">
+        <f aca="false">SUM(E2:E66)</f>
+        <v>36462.5</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
@@ -2415,6 +2447,11 @@
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Kadar: Konference 400 kg za 0,90 (presun z bloku Alexander Lucas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="114">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(47.6422225, 13.7605517) oder Konference (egal) – Menge noch offen – Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
@@ -480,7 +477,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,18 +523,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2208,33 +2193,36 @@
       <c r="H58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12" t="b">
-        <v>0</v>
-      </c>
+      <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G59" s="1"/>
+    </row>
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D59" s="1" t="n">
+      <c r="C60" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="D60" s="1" t="n">
         <v>0.9</v>
       </c>
-      <c r="E59" s="1" t="n">
-        <f aca="false">C59*D59</f>
-        <v>0</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="E60" s="1" t="n">
+        <f aca="false">C60*D60</f>
+        <v>360</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G59" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="H59" s="14"/>
-    </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="G60" s="1"/>
+      <c r="G60" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="b">
@@ -2262,7 +2250,7 @@
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2270,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C63" s="1" t="n">
         <v>400</v>
@@ -2283,17 +2271,17 @@
         <v>320</v>
       </c>
       <c r="F63" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G63" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G64" s="1"/>
     </row>
@@ -2345,7 +2333,7 @@
         <v>99</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H66" s="5" t="n">
         <v>46287</v>
@@ -2357,12 +2345,12 @@
       </c>
       <c r="C67" s="3" t="n">
         <f aca="false">SUM(C2:C66)</f>
-        <v>29498</v>
+        <v>29898</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="4" t="n">
         <f aca="false">SUM(E2:E66)</f>
-        <v>36462.5</v>
+        <v>36822.5</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2450,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Kadar: Konference 400 kg za 0,90 €/kg (#8)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="114">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(47.6422225, 13.7605517) oder Konference (egal) – Menge noch offen – Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
@@ -480,7 +477,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,18 +523,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2208,33 +2193,36 @@
       <c r="H58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12" t="b">
-        <v>0</v>
-      </c>
+      <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G59" s="1"/>
+    </row>
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D59" s="1" t="n">
+      <c r="C60" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="D60" s="1" t="n">
         <v>0.9</v>
       </c>
-      <c r="E59" s="1" t="n">
-        <f aca="false">C59*D59</f>
-        <v>0</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="E60" s="1" t="n">
+        <f aca="false">C60*D60</f>
+        <v>360</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G59" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="H59" s="14"/>
-    </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="G60" s="1"/>
+      <c r="G60" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="b">
@@ -2262,7 +2250,7 @@
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2270,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C63" s="1" t="n">
         <v>400</v>
@@ -2283,17 +2271,17 @@
         <v>320</v>
       </c>
       <c r="F63" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G63" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G64" s="1"/>
     </row>
@@ -2345,7 +2333,7 @@
         <v>99</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H66" s="5" t="n">
         <v>46287</v>
@@ -2357,12 +2345,12 @@
       </c>
       <c r="C67" s="3" t="n">
         <f aca="false">SUM(C2:C66)</f>
-        <v>29498</v>
+        <v>29898</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="4" t="n">
         <f aca="false">SUM(E2:E66)</f>
-        <v>36462.5</v>
+        <v>36822.5</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2450,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Nova objednavka: Martin Steinbichler, Amstetten, 300 kg Konference za 1,10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="116">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -344,6 +344,12 @@
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Martin Steinbichler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amstetten</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -477,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,6 +529,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,7 +801,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2249,91 +2263,86 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B62" s="1" t="s">
         <v>108</v>
       </c>
+      <c r="C62" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E62" s="1" t="n">
+        <f aca="false">C62*D62</f>
+        <v>330</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H62" s="13"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B63" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C63" s="1" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D63" s="1" t="n">
+      <c r="D64" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E63" s="1" t="n">
-        <f aca="false">C63*D63</f>
+      <c r="E64" s="1" t="n">
+        <f aca="false">C64*D64</f>
         <v>320</v>
       </c>
-      <c r="F63" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="H63" s="5"/>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1"/>
-      <c r="B64" s="1" t="s">
+      <c r="F64" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="G64" s="1"/>
+      <c r="G64" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A65" s="1"/>
       <c r="B65" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D65" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E65" s="1" t="n">
-        <f aca="false">C65*D65</f>
-        <v>240</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H65" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="G65" s="1"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C66" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D66" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E66" s="1" t="n">
         <f aca="false">C66*D66</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="H66" s="5" t="n">
         <v>46287</v>
@@ -2341,22 +2350,44 @@
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C67" s="3" t="n">
-        <f aca="false">SUM(C2:C66)</f>
-        <v>29898</v>
-      </c>
-      <c r="D67" s="3"/>
-      <c r="E67" s="4" t="n">
-        <f aca="false">SUM(E2:E66)</f>
-        <v>36822.5</v>
+        <v>1</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D67" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E67" s="1" t="n">
+        <f aca="false">C67*D67</f>
+        <v>225</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C68" s="3" t="n">
+        <f aca="false">SUM(C2:C67)</f>
+        <v>30198</v>
+      </c>
+      <c r="D68" s="3"/>
+      <c r="E68" s="4" t="n">
+        <f aca="false">SUM(E2:E67)</f>
+        <v>37152.5</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="b">
@@ -2440,6 +2471,11 @@
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nová objednávka: Martin Steinbichler, Amstetten – 300 kg Konference za 1,10 (#9)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="116">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -344,6 +344,12 @@
   </si>
   <si>
     <t xml:space="preserve">Birnen Konference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Martin Steinbichler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amstetten</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -477,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,6 +529,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,7 +801,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2249,91 +2263,86 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B62" s="1" t="s">
         <v>108</v>
       </c>
+      <c r="C62" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E62" s="1" t="n">
+        <f aca="false">C62*D62</f>
+        <v>330</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H62" s="13"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B63" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C63" s="1" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D63" s="1" t="n">
+      <c r="D64" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E63" s="1" t="n">
-        <f aca="false">C63*D63</f>
+      <c r="E64" s="1" t="n">
+        <f aca="false">C64*D64</f>
         <v>320</v>
       </c>
-      <c r="F63" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="H63" s="5"/>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1"/>
-      <c r="B64" s="1" t="s">
+      <c r="F64" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="G64" s="1"/>
+      <c r="G64" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A65" s="1"/>
       <c r="B65" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D65" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E65" s="1" t="n">
-        <f aca="false">C65*D65</f>
-        <v>240</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H65" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="G65" s="1"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C66" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D66" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E66" s="1" t="n">
         <f aca="false">C66*D66</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="H66" s="5" t="n">
         <v>46287</v>
@@ -2341,22 +2350,44 @@
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C67" s="3" t="n">
-        <f aca="false">SUM(C2:C66)</f>
-        <v>29898</v>
-      </c>
-      <c r="D67" s="3"/>
-      <c r="E67" s="4" t="n">
-        <f aca="false">SUM(E2:E66)</f>
-        <v>36822.5</v>
+        <v>1</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D67" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E67" s="1" t="n">
+        <f aca="false">C67*D67</f>
+        <v>225</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C68" s="3" t="n">
+        <f aca="false">SUM(C2:C67)</f>
+        <v>30198</v>
+      </c>
+      <c r="D68" s="3"/>
+      <c r="E68" s="4" t="n">
+        <f aca="false">SUM(E2:E67)</f>
+        <v>37152.5</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="b">
@@ -2440,6 +2471,11 @@
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Steinbichler: presna adresa Kuglau 93, 3361 Biberbach
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -349,7 +349,7 @@
     <t xml:space="preserve">Martin Steinbichler</t>
   </si>
   <si>
-    <t xml:space="preserve">Amstetten</t>
+    <t xml:space="preserve">Kuglau 93, 3361 Biberbach</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -483,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,14 +529,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2263,7 +2255,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12" t="b">
+      <c r="A62" s="11" t="b">
         <v>0</v>
       </c>
       <c r="B62" s="1" t="s">
@@ -2282,7 +2274,7 @@
       <c r="F62" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="H62" s="13"/>
+      <c r="H62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="1" t="s">
@@ -2474,7 +2466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Steinbichler: přesná adresa Kuglau 93, 3361 Biberbach (#10)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -349,7 +349,7 @@
     <t xml:space="preserve">Martin Steinbichler</t>
   </si>
   <si>
-    <t xml:space="preserve">Amstetten</t>
+    <t xml:space="preserve">Kuglau 93, 3361 Biberbach</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -483,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,14 +529,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2263,7 +2255,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12" t="b">
+      <c r="A62" s="11" t="b">
         <v>0</v>
       </c>
       <c r="B62" s="1" t="s">
@@ -2282,7 +2274,7 @@
       <c r="F62" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="H62" s="13"/>
+      <c r="H62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="1" t="s">
@@ -2474,7 +2466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Doruceno 3.10.: Kadar 420 kg Konference za 0,90 + 380 kg Williams za 1,20, Gasteiger 500 Konference + 500 Lucas za 0,90, Franz Huber 320 kg Konference za 0,90 (adresa chybi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="117">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -304,7 +304,7 @@
     <t xml:space="preserve">Abholung in Salzburg oder Radstadt möglich – pauschal 700 €</t>
   </si>
   <si>
-    <t xml:space="preserve">(47.6422225, 13.7605517) Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
+    <t xml:space="preserve">(47.6422225, 13.7605517)</t>
   </si>
   <si>
     <t xml:space="preserve">Gerhard Bayer</t>
@@ -340,9 +340,6 @@
     <t xml:space="preserve">Birnen Alexander Lucas</t>
   </si>
   <si>
-    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
-  </si>
-  <si>
     <t xml:space="preserve">Birnen Konference</t>
   </si>
   <si>
@@ -350,6 +347,12 @@
   </si>
   <si>
     <t xml:space="preserve">Kuglau 93, 3361 Biberbach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Franz Huber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adresse fehlt</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -483,7 +486,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,6 +532,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -793,7 +808,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2013,26 +2028,29 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C50" s="1" t="n">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="D50" s="1" t="n">
         <v>1.2</v>
       </c>
       <c r="E50" s="1" t="n">
         <f aca="false">C50*D50</f>
-        <v>480</v>
+        <v>456</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>94</v>
+      </c>
+      <c r="H50" s="12" t="n">
+        <v>46298</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2175,7 +2193,7 @@
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>43</v>
@@ -2184,43 +2202,43 @@
         <v>500</v>
       </c>
       <c r="D58" s="1" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="E58" s="1" t="n">
         <f aca="false">C58*D58</f>
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G58" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H58" s="5"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G59" s="1"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C60" s="1" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="D60" s="1" t="n">
         <v>0.9</v>
       </c>
       <c r="E60" s="1" t="n">
         <f aca="false">C60*D60</f>
-        <v>360</v>
+        <v>378</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>23</v>
@@ -2228,11 +2246,13 @@
       <c r="G60" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H60" s="5"/>
+      <c r="H60" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>43</v>
@@ -2241,17 +2261,18 @@
         <v>500</v>
       </c>
       <c r="D61" s="1" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="E61" s="1" t="n">
         <f aca="false">C61*D61</f>
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G61" s="1" t="s">
-        <v>106</v>
+      <c r="G61" s="1"/>
+      <c r="H61" s="12" t="n">
+        <v>46298</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2259,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C62" s="1" t="n">
         <v>300</v>
@@ -2272,96 +2293,93 @@
         <v>330</v>
       </c>
       <c r="F62" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="H62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B63" s="1" t="s">
+      <c r="C63" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="D63" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E63" s="1" t="n">
+        <f aca="false">C63*D63</f>
+        <v>288</v>
+      </c>
+      <c r="G63" s="14" t="s">
         <v>110</v>
       </c>
+      <c r="H63" s="12" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B64" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C64" s="1" t="n">
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D64" s="1" t="n">
+      <c r="D65" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E64" s="1" t="n">
-        <f aca="false">C64*D64</f>
+      <c r="E65" s="1" t="n">
+        <f aca="false">C65*D65</f>
         <v>320</v>
       </c>
-      <c r="F64" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="G64" s="1" t="s">
+      <c r="F65" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="H64" s="5"/>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1"/>
-      <c r="B65" s="1" t="s">
+      <c r="G65" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="G65" s="1"/>
+      <c r="H65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A66" s="1"/>
       <c r="B66" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D66" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E66" s="1" t="n">
-        <f aca="false">C66*D66</f>
-        <v>240</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H66" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G66" s="1"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C67" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D67" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E67" s="1" t="n">
         <f aca="false">C67*D67</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="H67" s="5" t="n">
         <v>46287</v>
@@ -2369,22 +2387,44 @@
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C68" s="3" t="n">
-        <f aca="false">SUM(C2:C67)</f>
-        <v>30198</v>
-      </c>
-      <c r="D68" s="3"/>
-      <c r="E68" s="4" t="n">
-        <f aca="false">SUM(E2:E67)</f>
-        <v>37152.5</v>
+        <v>1</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C68" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D68" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E68" s="1" t="n">
+        <f aca="false">C68*D68</f>
+        <v>225</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="H68" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C69" s="3" t="n">
+        <f aca="false">SUM(C2:C68)</f>
+        <v>30518</v>
+      </c>
+      <c r="D69" s="3"/>
+      <c r="E69" s="4" t="n">
+        <f aca="false">SUM(E2:E68)</f>
+        <v>37384.5</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="11" t="b">
@@ -2468,6 +2508,11 @@
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Doručeno 3. 10.: Kadar, Gasteiger, Franz Huber (#11)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="117">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -304,7 +304,7 @@
     <t xml:space="preserve">Abholung in Salzburg oder Radstadt möglich – pauschal 700 €</t>
   </si>
   <si>
-    <t xml:space="preserve">(47.6422225, 13.7605517) Kunde erst ab So 4.10. mittags da – Abladen auch ohne ihn möglich</t>
+    <t xml:space="preserve">(47.6422225, 13.7605517)</t>
   </si>
   <si>
     <t xml:space="preserve">Gerhard Bayer</t>
@@ -340,9 +340,6 @@
     <t xml:space="preserve">Birnen Alexander Lucas</t>
   </si>
   <si>
-    <t xml:space="preserve">Lieferung am liebsten Sa 3.10. abends</t>
-  </si>
-  <si>
     <t xml:space="preserve">Birnen Konference</t>
   </si>
   <si>
@@ -350,6 +347,12 @@
   </si>
   <si>
     <t xml:space="preserve">Kuglau 93, 3361 Biberbach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Franz Huber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adresse fehlt</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -483,7 +486,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,6 +532,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -793,7 +808,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2013,26 +2028,29 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C50" s="1" t="n">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="D50" s="1" t="n">
         <v>1.2</v>
       </c>
       <c r="E50" s="1" t="n">
         <f aca="false">C50*D50</f>
-        <v>480</v>
+        <v>456</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>94</v>
+      </c>
+      <c r="H50" s="12" t="n">
+        <v>46298</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2175,7 +2193,7 @@
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>43</v>
@@ -2184,43 +2202,43 @@
         <v>500</v>
       </c>
       <c r="D58" s="1" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="E58" s="1" t="n">
         <f aca="false">C58*D58</f>
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G58" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H58" s="5"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G59" s="1"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C60" s="1" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="D60" s="1" t="n">
         <v>0.9</v>
       </c>
       <c r="E60" s="1" t="n">
         <f aca="false">C60*D60</f>
-        <v>360</v>
+        <v>378</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>23</v>
@@ -2228,11 +2246,13 @@
       <c r="G60" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H60" s="5"/>
+      <c r="H60" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>43</v>
@@ -2241,17 +2261,18 @@
         <v>500</v>
       </c>
       <c r="D61" s="1" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="E61" s="1" t="n">
         <f aca="false">C61*D61</f>
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G61" s="1" t="s">
-        <v>106</v>
+      <c r="G61" s="1"/>
+      <c r="H61" s="12" t="n">
+        <v>46298</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2259,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C62" s="1" t="n">
         <v>300</v>
@@ -2272,96 +2293,93 @@
         <v>330</v>
       </c>
       <c r="F62" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="H62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B63" s="1" t="s">
+      <c r="C63" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="D63" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E63" s="1" t="n">
+        <f aca="false">C63*D63</f>
+        <v>288</v>
+      </c>
+      <c r="G63" s="14" t="s">
         <v>110</v>
       </c>
+      <c r="H63" s="12" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B64" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C64" s="1" t="n">
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="D64" s="1" t="n">
+      <c r="D65" s="1" t="n">
         <v>0.8</v>
       </c>
-      <c r="E64" s="1" t="n">
-        <f aca="false">C64*D64</f>
+      <c r="E65" s="1" t="n">
+        <f aca="false">C65*D65</f>
         <v>320</v>
       </c>
-      <c r="F64" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="G64" s="1" t="s">
+      <c r="F65" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="H64" s="5"/>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1"/>
-      <c r="B65" s="1" t="s">
+      <c r="G65" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="G65" s="1"/>
+      <c r="H65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A66" s="1"/>
       <c r="B66" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D66" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E66" s="1" t="n">
-        <f aca="false">C66*D66</f>
-        <v>240</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H66" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G66" s="1"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C67" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D67" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E67" s="1" t="n">
         <f aca="false">C67*D67</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="H67" s="5" t="n">
         <v>46287</v>
@@ -2369,22 +2387,44 @@
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C68" s="3" t="n">
-        <f aca="false">SUM(C2:C67)</f>
-        <v>30198</v>
-      </c>
-      <c r="D68" s="3"/>
-      <c r="E68" s="4" t="n">
-        <f aca="false">SUM(E2:E67)</f>
-        <v>37152.5</v>
+        <v>1</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C68" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D68" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E68" s="1" t="n">
+        <f aca="false">C68*D68</f>
+        <v>225</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="H68" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C69" s="3" t="n">
+        <f aca="false">SUM(C2:C68)</f>
+        <v>30518</v>
+      </c>
+      <c r="D69" s="3"/>
+      <c r="E69" s="4" t="n">
+        <f aca="false">SUM(E2:E68)</f>
+        <v>37384.5</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="11" t="b">
@@ -2468,6 +2508,11 @@
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Franz Huber: adresa Emming 4, 4892 Fornach (Huber's Edelbrände), telefon z vizitky
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="118">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -352,7 +352,10 @@
     <t xml:space="preserve">Franz Huber</t>
   </si>
   <si>
-    <t xml:space="preserve">Adresse fehlt</t>
+    <t xml:space="preserve">Emming 4, 4892 Fornach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huber's Edelbrände, Tel. +43 677/62392405</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -486,7 +489,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -532,18 +535,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2049,7 +2040,7 @@
       <c r="G50" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H50" s="12" t="n">
+      <c r="H50" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
@@ -2271,7 +2262,7 @@
         <v>44</v>
       </c>
       <c r="G61" s="1"/>
-      <c r="H61" s="12" t="n">
+      <c r="H61" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
@@ -2298,7 +2289,7 @@
       <c r="H62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="13" t="b">
+      <c r="A63" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B63" s="1" t="s">
@@ -2314,16 +2305,19 @@
         <f aca="false">C63*D63</f>
         <v>288</v>
       </c>
-      <c r="G63" s="14" t="s">
+      <c r="F63" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="H63" s="12" t="n">
+      <c r="G63" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H63" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2331,7 +2325,7 @@
         <v>0</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C65" s="1" t="n">
         <v>400</v>
@@ -2344,17 +2338,17 @@
         <v>320</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1"/>
       <c r="B66" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G66" s="1"/>
     </row>
@@ -2406,7 +2400,7 @@
         <v>99</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H68" s="5" t="n">
         <v>46287</v>
@@ -2511,7 +2505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Franz Huber: adresa Emming 4, 4892 Fornach (#12)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="118">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -352,7 +352,10 @@
     <t xml:space="preserve">Franz Huber</t>
   </si>
   <si>
-    <t xml:space="preserve">Adresse fehlt</t>
+    <t xml:space="preserve">Emming 4, 4892 Fornach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huber's Edelbrände, Tel. +43 677/62392405</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen</t>
@@ -486,7 +489,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -532,18 +535,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2049,7 +2040,7 @@
       <c r="G50" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H50" s="12" t="n">
+      <c r="H50" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
@@ -2271,7 +2262,7 @@
         <v>44</v>
       </c>
       <c r="G61" s="1"/>
-      <c r="H61" s="12" t="n">
+      <c r="H61" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
@@ -2298,7 +2289,7 @@
       <c r="H62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="13" t="b">
+      <c r="A63" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B63" s="1" t="s">
@@ -2314,16 +2305,19 @@
         <f aca="false">C63*D63</f>
         <v>288</v>
       </c>
-      <c r="G63" s="14" t="s">
+      <c r="F63" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="H63" s="12" t="n">
+      <c r="G63" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H63" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2331,7 +2325,7 @@
         <v>0</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C65" s="1" t="n">
         <v>400</v>
@@ -2344,17 +2338,17 @@
         <v>320</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1"/>
       <c r="B66" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G66" s="1"/>
     </row>
@@ -2406,7 +2400,7 @@
         <v>99</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H68" s="5" t="n">
         <v>46287</v>
@@ -2511,7 +2505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Doruceno 6.10.: Moser 800 kg Alexander Lucas za 0,80 (misto objednanych 1000 kg)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -489,7 +489,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,6 +535,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2162,25 +2166,28 @@
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="D57" s="1" t="n">
         <v>0.8</v>
       </c>
       <c r="E57" s="1" t="n">
         <f aca="false">C57*D57</f>
-        <v>800</v>
+        <v>640</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>31</v>
       </c>
       <c r="G57" s="1"/>
+      <c r="H57" s="12" t="n">
+        <v>46301</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="b">
@@ -2412,12 +2419,12 @@
       </c>
       <c r="C69" s="3" t="n">
         <f aca="false">SUM(C2:C68)</f>
-        <v>30518</v>
+        <v>30318</v>
       </c>
       <c r="D69" s="3"/>
       <c r="E69" s="4" t="n">
         <f aca="false">SUM(E2:E68)</f>
-        <v>37384.5</v>
+        <v>37224.5</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Doručeno 6. 10.: Moser 800 kg Alexander Lucas za 0,80 (#15)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -489,7 +489,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,6 +535,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2162,25 +2166,28 @@
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="D57" s="1" t="n">
         <v>0.8</v>
       </c>
       <c r="E57" s="1" t="n">
         <f aca="false">C57*D57</f>
-        <v>800</v>
+        <v>640</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>31</v>
       </c>
       <c r="G57" s="1"/>
+      <c r="H57" s="12" t="n">
+        <v>46301</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="b">
@@ -2412,12 +2419,12 @@
       </c>
       <c r="C69" s="3" t="n">
         <f aca="false">SUM(C2:C68)</f>
-        <v>30518</v>
+        <v>30318</v>
       </c>
       <c r="D69" s="3"/>
       <c r="E69" s="4" t="n">
         <f aca="false">SUM(E2:E68)</f>
-        <v>37384.5</v>
+        <v>37224.5</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Nova objednavka: Martin Neuwirth 400 kg Packham za 1 EUR/kg, odber ve Spittalu (zatim nepotvrzeno)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="121">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -335,6 +335,15 @@
   </si>
   <si>
     <t xml:space="preserve">Birnen Packham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Martin Neuwirth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spittal an der Drau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abholung in Spittal an der Drau – Kunde aus 9634 Gundersheim – für Saft und Most – 1 €/kg bei Abholung angeboten, Zusage offen</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Alexander Lucas</t>
@@ -489,7 +498,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,6 +544,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -803,7 +820,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2158,256 +2175,254 @@
       <c r="G55" s="1"/>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1"/>
+      <c r="A56" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B56" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="G56" s="1"/>
+      <c r="C56" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="D56" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="1" t="n">
+        <f aca="false">C56*D56</f>
+        <v>400</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G56" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="H56" s="14"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A57" s="1"/>
       <c r="B57" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C57" s="1" t="n">
-        <v>800</v>
-      </c>
-      <c r="D57" s="1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E57" s="1" t="n">
-        <f aca="false">C57*D57</f>
-        <v>640</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>31</v>
+        <v>108</v>
       </c>
       <c r="G57" s="1"/>
-      <c r="H57" s="12" t="n">
-        <v>46301</v>
-      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="C58" s="1" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="D58" s="1" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E58" s="1" t="n">
         <f aca="false">C58*D58</f>
-        <v>450</v>
+        <v>640</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" s="5" t="n">
+        <v>46301</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <f aca="false">C59*D59</f>
+        <v>450</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G59" s="1"/>
+      <c r="H59" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G59" s="1"/>
-    </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C60" s="1" t="n">
-        <v>420</v>
-      </c>
-      <c r="D60" s="1" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E60" s="1" t="n">
-        <f aca="false">C60*D60</f>
-        <v>378</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H60" s="5" t="n">
-        <v>46298</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="G60" s="1"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="C61" s="1" t="n">
-        <v>500</v>
+        <v>420</v>
       </c>
       <c r="D61" s="1" t="n">
         <v>0.9</v>
       </c>
       <c r="E61" s="1" t="n">
         <f aca="false">C61*D61</f>
-        <v>450</v>
+        <v>378</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G61" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="H61" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="C62" s="1" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D62" s="1" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E62" s="1" t="n">
         <f aca="false">C62*D62</f>
-        <v>330</v>
+        <v>450</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H62" s="5"/>
+        <v>44</v>
+      </c>
+      <c r="G62" s="1"/>
+      <c r="H62" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C63" s="1" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="D63" s="1" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E63" s="1" t="n">
         <f aca="false">C63*D63</f>
-        <v>288</v>
+        <v>330</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G63" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H63" s="5" t="n">
-        <v>46298</v>
-      </c>
+      <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="b">
+        <v>1</v>
+      </c>
       <c r="B64" s="1" t="s">
         <v>112</v>
       </c>
+      <c r="C64" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="D64" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E64" s="1" t="n">
+        <f aca="false">C64*D64</f>
+        <v>288</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H64" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B65" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D65" s="1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E65" s="1" t="n">
-        <f aca="false">C65*D65</f>
-        <v>320</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G65" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="H65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1"/>
+      <c r="A66" s="11" t="b">
+        <v>0</v>
+      </c>
       <c r="B66" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G66" s="1"/>
+      <c r="C66" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E66" s="1" t="n">
+        <f aca="false">C66*D66</f>
+        <v>320</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D67" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E67" s="1" t="n">
-        <f aca="false">C67*D67</f>
-        <v>240</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H67" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="G67" s="1"/>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C68" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D68" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E68" s="1" t="n">
         <f aca="false">C68*D68</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="H68" s="5" t="n">
         <v>46287</v>
@@ -2415,22 +2430,44 @@
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C69" s="3" t="n">
-        <f aca="false">SUM(C2:C68)</f>
-        <v>30318</v>
-      </c>
-      <c r="D69" s="3"/>
-      <c r="E69" s="4" t="n">
-        <f aca="false">SUM(E2:E68)</f>
-        <v>37224.5</v>
+        <v>1</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C69" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E69" s="1" t="n">
+        <f aca="false">C69*D69</f>
+        <v>225</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H69" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C70" s="3" t="n">
+        <f aca="false">SUM(C2:C69)</f>
+        <v>30718</v>
+      </c>
+      <c r="D70" s="3"/>
+      <c r="E70" s="4" t="n">
+        <f aca="false">SUM(E2:E69)</f>
+        <v>37624.5</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="b">
@@ -2514,6 +2551,11 @@
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nová objednávka: Martin Neuwirth – 400 kg Packham, odběr Spittal (#17)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="121">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -335,6 +335,15 @@
   </si>
   <si>
     <t xml:space="preserve">Birnen Packham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Martin Neuwirth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spittal an der Drau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abholung in Spittal an der Drau – Kunde aus 9634 Gundersheim – für Saft und Most – 1 €/kg bei Abholung angeboten, Zusage offen</t>
   </si>
   <si>
     <t xml:space="preserve">Birnen Alexander Lucas</t>
@@ -489,7 +498,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,6 +544,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -803,7 +820,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="10.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
@@ -2158,256 +2175,254 @@
       <c r="G55" s="1"/>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1"/>
+      <c r="A56" s="12" t="b">
+        <v>0</v>
+      </c>
       <c r="B56" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="G56" s="1"/>
+      <c r="C56" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="D56" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="1" t="n">
+        <f aca="false">C56*D56</f>
+        <v>400</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G56" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="H56" s="14"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A57" s="1"/>
       <c r="B57" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C57" s="1" t="n">
-        <v>800</v>
-      </c>
-      <c r="D57" s="1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E57" s="1" t="n">
-        <f aca="false">C57*D57</f>
-        <v>640</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>31</v>
+        <v>108</v>
       </c>
       <c r="G57" s="1"/>
-      <c r="H57" s="12" t="n">
-        <v>46301</v>
-      </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="C58" s="1" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="D58" s="1" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E58" s="1" t="n">
         <f aca="false">C58*D58</f>
-        <v>450</v>
+        <v>640</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" s="5" t="n">
+        <v>46301</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <f aca="false">C59*D59</f>
+        <v>450</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G59" s="1"/>
+      <c r="H59" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G59" s="1"/>
-    </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C60" s="1" t="n">
-        <v>420</v>
-      </c>
-      <c r="D60" s="1" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E60" s="1" t="n">
-        <f aca="false">C60*D60</f>
-        <v>378</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H60" s="5" t="n">
-        <v>46298</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="G60" s="1"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="C61" s="1" t="n">
-        <v>500</v>
+        <v>420</v>
       </c>
       <c r="D61" s="1" t="n">
         <v>0.9</v>
       </c>
       <c r="E61" s="1" t="n">
         <f aca="false">C61*D61</f>
-        <v>450</v>
+        <v>378</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G61" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="H61" s="5" t="n">
         <v>46298</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="C62" s="1" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D62" s="1" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E62" s="1" t="n">
         <f aca="false">C62*D62</f>
-        <v>330</v>
+        <v>450</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H62" s="5"/>
+        <v>44</v>
+      </c>
+      <c r="G62" s="1"/>
+      <c r="H62" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C63" s="1" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="D63" s="1" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E63" s="1" t="n">
         <f aca="false">C63*D63</f>
-        <v>288</v>
+        <v>330</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G63" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H63" s="5" t="n">
-        <v>46298</v>
-      </c>
+      <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="b">
+        <v>1</v>
+      </c>
       <c r="B64" s="1" t="s">
         <v>112</v>
       </c>
+      <c r="C64" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="D64" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E64" s="1" t="n">
+        <f aca="false">C64*D64</f>
+        <v>288</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H64" s="5" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="11" t="b">
-        <v>0</v>
-      </c>
       <c r="B65" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D65" s="1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E65" s="1" t="n">
-        <f aca="false">C65*D65</f>
-        <v>320</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G65" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="H65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1"/>
+      <c r="A66" s="11" t="b">
+        <v>0</v>
+      </c>
       <c r="B66" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G66" s="1"/>
+      <c r="C66" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E66" s="1" t="n">
+        <f aca="false">C66*D66</f>
+        <v>320</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="11" t="b">
-        <v>1</v>
-      </c>
+      <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>400</v>
-      </c>
-      <c r="D67" s="1" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E67" s="1" t="n">
-        <f aca="false">C67*D67</f>
-        <v>240</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H67" s="5" t="n">
-        <v>46287</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="G67" s="1"/>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="b">
         <v>1</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C68" s="1" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D68" s="1" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="E68" s="1" t="n">
         <f aca="false">C68*D68</f>
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="H68" s="5" t="n">
         <v>46287</v>
@@ -2415,22 +2430,44 @@
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C69" s="3" t="n">
-        <f aca="false">SUM(C2:C68)</f>
-        <v>30318</v>
-      </c>
-      <c r="D69" s="3"/>
-      <c r="E69" s="4" t="n">
-        <f aca="false">SUM(E2:E68)</f>
-        <v>37224.5</v>
+        <v>1</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C69" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E69" s="1" t="n">
+        <f aca="false">C69*D69</f>
+        <v>225</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H69" s="5" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="11" t="b">
         <v>0</v>
       </c>
+      <c r="C70" s="3" t="n">
+        <f aca="false">SUM(C2:C69)</f>
+        <v>30718</v>
+      </c>
+      <c r="D70" s="3"/>
+      <c r="E70" s="4" t="n">
+        <f aca="false">SUM(E2:E69)</f>
+        <v>37624.5</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="b">
@@ -2514,6 +2551,11 @@
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Burgstaller: 26.-30.10. pryc, dovoz az od 31.10.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t xml:space="preserve">Birnen Packham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urlaub 26.10.–30.10. – Lieferung erst danach (ab 31.10.)</t>
   </si>
   <si>
     <t xml:space="preserve">Martin Neuwirth</t>
@@ -498,7 +501,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -544,18 +547,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2172,14 +2163,16 @@
       <c r="F55" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G55" s="1"/>
+      <c r="G55" s="1" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12" t="b">
+      <c r="A56" s="11" t="b">
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C56" s="1" t="n">
         <v>400</v>
@@ -2192,17 +2185,17 @@
         <v>400</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G56" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="H56" s="14"/>
+      <c r="G56" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1"/>
       <c r="B57" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G57" s="1"/>
     </row>
@@ -2259,7 +2252,7 @@
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G60" s="1"/>
     </row>
@@ -2320,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C63" s="1" t="n">
         <v>300</v>
@@ -2333,7 +2326,7 @@
         <v>330</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H63" s="5"/>
     </row>
@@ -2342,7 +2335,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C64" s="1" t="n">
         <v>320</v>
@@ -2355,10 +2348,10 @@
         <v>288</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>46298</v>
@@ -2366,7 +2359,7 @@
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2374,7 +2367,7 @@
         <v>0</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C66" s="1" t="n">
         <v>400</v>
@@ -2387,17 +2380,17 @@
         <v>320</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G67" s="1"/>
     </row>
@@ -2449,7 +2442,7 @@
         <v>99</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H69" s="5" t="n">
         <v>46287</v>
@@ -2554,7 +2547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Burgstaller: 26.–30. 10. pryč, dovoz až od 31. 10. (#18)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t xml:space="preserve">Birnen Packham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urlaub 26.10.–30.10. – Lieferung erst danach (ab 31.10.)</t>
   </si>
   <si>
     <t xml:space="preserve">Martin Neuwirth</t>
@@ -498,7 +501,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -544,18 +547,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2172,14 +2163,16 @@
       <c r="F55" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G55" s="1"/>
+      <c r="G55" s="1" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12" t="b">
+      <c r="A56" s="11" t="b">
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C56" s="1" t="n">
         <v>400</v>
@@ -2192,17 +2185,17 @@
         <v>400</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G56" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="H56" s="14"/>
+      <c r="G56" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1"/>
       <c r="B57" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G57" s="1"/>
     </row>
@@ -2259,7 +2252,7 @@
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G60" s="1"/>
     </row>
@@ -2320,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C63" s="1" t="n">
         <v>300</v>
@@ -2333,7 +2326,7 @@
         <v>330</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H63" s="5"/>
     </row>
@@ -2342,7 +2335,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C64" s="1" t="n">
         <v>320</v>
@@ -2355,10 +2348,10 @@
         <v>288</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>46298</v>
@@ -2366,7 +2359,7 @@
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2374,7 +2367,7 @@
         <v>0</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C66" s="1" t="n">
         <v>400</v>
@@ -2387,17 +2380,17 @@
         <v>320</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G67" s="1"/>
     </row>
@@ -2449,7 +2442,7 @@
         <v>99</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H69" s="5" t="n">
         <v>46287</v>
@@ -2554,7 +2547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Steinbichler zrusen (neozval se) - STORNIERT, mnozstvi 0, kontakt zustava
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="123">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -359,6 +359,9 @@
   </si>
   <si>
     <t xml:space="preserve">Kuglau 93, 3361 Biberbach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STORNIERT 2026 – Kunde hat sich nicht mehr gemeldet – ursprünglich 300 kg à 1,10</t>
   </si>
   <si>
     <t xml:space="preserve">Franz Huber</t>
@@ -501,7 +504,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -547,6 +550,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2316,18 +2323,21 @@
         <v>111</v>
       </c>
       <c r="C63" s="1" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="D63" s="1" t="n">
         <v>1.1</v>
       </c>
       <c r="E63" s="1" t="n">
         <f aca="false">C63*D63</f>
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>112</v>
       </c>
+      <c r="G63" s="12" t="s">
+        <v>113</v>
+      </c>
       <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C64" s="1" t="n">
         <v>320</v>
@@ -2348,10 +2358,10 @@
         <v>288</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>46298</v>
@@ -2359,7 +2369,7 @@
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2367,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C66" s="1" t="n">
         <v>400</v>
@@ -2380,17 +2390,17 @@
         <v>320</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G67" s="1"/>
     </row>
@@ -2442,7 +2452,7 @@
         <v>99</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H69" s="5" t="n">
         <v>46287</v>
@@ -2454,12 +2464,12 @@
       </c>
       <c r="C70" s="3" t="n">
         <f aca="false">SUM(C2:C69)</f>
-        <v>30718</v>
+        <v>30418</v>
       </c>
       <c r="D70" s="3"/>
       <c r="E70" s="4" t="n">
         <f aca="false">SUM(E2:E69)</f>
-        <v>37624.5</v>
+        <v>37294.5</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Steinbichler zrušen – neozval se (#19)
Claude-Session: https://claude.ai/code/session_01EHrNoviFMMThbs95mXweRJ

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="123">
   <si>
     <t xml:space="preserve">Geliefert</t>
   </si>
@@ -359,6 +359,9 @@
   </si>
   <si>
     <t xml:space="preserve">Kuglau 93, 3361 Biberbach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STORNIERT 2026 – Kunde hat sich nicht mehr gemeldet – ursprünglich 300 kg à 1,10</t>
   </si>
   <si>
     <t xml:space="preserve">Franz Huber</t>
@@ -501,7 +504,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -547,6 +550,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2316,18 +2323,21 @@
         <v>111</v>
       </c>
       <c r="C63" s="1" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="D63" s="1" t="n">
         <v>1.1</v>
       </c>
       <c r="E63" s="1" t="n">
         <f aca="false">C63*D63</f>
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>112</v>
       </c>
+      <c r="G63" s="12" t="s">
+        <v>113</v>
+      </c>
       <c r="H63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C64" s="1" t="n">
         <v>320</v>
@@ -2348,10 +2358,10 @@
         <v>288</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>46298</v>
@@ -2359,7 +2369,7 @@
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2367,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C66" s="1" t="n">
         <v>400</v>
@@ -2380,17 +2390,17 @@
         <v>320</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G67" s="1"/>
     </row>
@@ -2442,7 +2452,7 @@
         <v>99</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H69" s="5" t="n">
         <v>46287</v>
@@ -2454,12 +2464,12 @@
       </c>
       <c r="C70" s="3" t="n">
         <f aca="false">SUM(C2:C69)</f>
-        <v>30718</v>
+        <v>30418</v>
       </c>
       <c r="D70" s="3"/>
       <c r="E70" s="4" t="n">
         <f aca="false">SUM(E2:E69)</f>
-        <v>37624.5</v>
+        <v>37294.5</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>